<commit_message>
data: atualiza planilha CONTAS-A-RECEBER.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docx_templates/CONTAS-A-RECEBER.xlsx
+++ b/docx_templates/CONTAS-A-RECEBER.xlsx
@@ -9,14 +9,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Relatório!$A$5:$S$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$68</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -103,340 +103,334 @@
     <t>1.0 [OFICIAL] SICREDI | BANCO GESTOR</t>
   </si>
   <si>
+    <t>VENCIDO ATÉ 30 DIAS</t>
+  </si>
+  <si>
+    <t>FA-11240</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DIEGO TAYAO DANTAS</t>
+  </si>
+  <si>
+    <t>VENCIDO</t>
+  </si>
+  <si>
+    <t>FATURA</t>
+  </si>
+  <si>
+    <t>ATIVUZ VEÍCULOS</t>
+  </si>
+  <si>
+    <t>VENCIDO ENTRE 31 A 90 DIAS</t>
+  </si>
+  <si>
+    <t>FA-11155</t>
+  </si>
+  <si>
+    <t>OLIZIEL DA SILVA CARDOSO</t>
+  </si>
+  <si>
+    <t>FA-11496</t>
+  </si>
+  <si>
+    <t>ANDRE CAVALCANTI DA FE</t>
+  </si>
+  <si>
+    <t>AZ EMPREENDIMENTOS</t>
+  </si>
+  <si>
+    <t>FA-11447</t>
+  </si>
+  <si>
+    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
+  </si>
+  <si>
+    <t>FA-11421</t>
+  </si>
+  <si>
+    <t>FA-11255</t>
+  </si>
+  <si>
+    <t>LEONARDO GOMES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11406</t>
+  </si>
+  <si>
+    <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11383</t>
+  </si>
+  <si>
+    <t>JOZILDO TARQUINO DE BRITO</t>
+  </si>
+  <si>
+    <t>FA-11419</t>
+  </si>
+  <si>
+    <t>YURI BATISTA DA COSTA</t>
+  </si>
+  <si>
+    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11189</t>
+  </si>
+  <si>
+    <t>FA-11182</t>
+  </si>
+  <si>
+    <t>MARCELO BENTO DE ARAUJO</t>
+  </si>
+  <si>
+    <t>FA-11069</t>
+  </si>
+  <si>
+    <t>ALBERTO MANOEL DOS REIS</t>
+  </si>
+  <si>
+    <t>PRIVADO</t>
+  </si>
+  <si>
+    <t>ND-11305</t>
+  </si>
+  <si>
+    <t>NOTA DE DÉBITO</t>
+  </si>
+  <si>
+    <t>FA-11113</t>
+  </si>
+  <si>
+    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
+  </si>
+  <si>
     <t>VENCIDO ACIMA DE 90 DIAS</t>
   </si>
   <si>
-    <t>ND-11056</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>LENILDO DE LIMA</t>
-  </si>
-  <si>
-    <t>VENCIDO</t>
-  </si>
-  <si>
-    <t>NOTA DE DÉBITO</t>
-  </si>
-  <si>
-    <t>ATIVUZ VEÍCULOS</t>
-  </si>
-  <si>
-    <t>VENCIDO ENTRE 31 A 90 DIAS</t>
+    <t>ND-10427</t>
+  </si>
+  <si>
+    <t>RICARDO ARAUJO DE MIRANDA</t>
+  </si>
+  <si>
+    <t>FA-11455</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11426</t>
+  </si>
+  <si>
+    <t>FA-11244</t>
+  </si>
+  <si>
+    <t>FA-11390</t>
+  </si>
+  <si>
+    <t>ADRIANO SANTOS DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
+  </si>
+  <si>
+    <t>FA-11115</t>
+  </si>
+  <si>
+    <t>FA-11256</t>
+  </si>
+  <si>
+    <t>FA-11424</t>
+  </si>
+  <si>
+    <t>FA-11407</t>
+  </si>
+  <si>
+    <t>FA-11183</t>
+  </si>
+  <si>
+    <t>FA-11361</t>
+  </si>
+  <si>
+    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
+  </si>
+  <si>
+    <t>FA-11452</t>
+  </si>
+  <si>
+    <t>YAGO ELIAS COSTA BATISTA</t>
+  </si>
+  <si>
+    <t>FA-11346</t>
+  </si>
+  <si>
+    <t>FA-11114</t>
+  </si>
+  <si>
+    <t>FA-11456</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11253</t>
+  </si>
+  <si>
+    <t>HOJE</t>
+  </si>
+  <si>
+    <t>FA-11387</t>
+  </si>
+  <si>
+    <t>A VENCER</t>
+  </si>
+  <si>
+    <t>FA-11147</t>
+  </si>
+  <si>
+    <t>FA-11458</t>
+  </si>
+  <si>
+    <t>FA-11392</t>
+  </si>
+  <si>
+    <t>FA-11516</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11462</t>
+  </si>
+  <si>
+    <t>FA-11153</t>
+  </si>
+  <si>
+    <t>FA-11393</t>
+  </si>
+  <si>
+    <t>FA-11351</t>
+  </si>
+  <si>
+    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11350</t>
+  </si>
+  <si>
+    <t>FA-11391</t>
+  </si>
+  <si>
+    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
+  </si>
+  <si>
+    <t>FA-11485</t>
+  </si>
+  <si>
+    <t>ROSSILY PEREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11517</t>
+  </si>
+  <si>
+    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11500</t>
+  </si>
+  <si>
+    <t>WESCLY JEAN DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>FA-11497</t>
+  </si>
+  <si>
+    <t>FA-11460</t>
+  </si>
+  <si>
+    <t>FA-11369</t>
+  </si>
+  <si>
+    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>FA-11111</t>
+  </si>
+  <si>
+    <t>FA-11276</t>
+  </si>
+  <si>
+    <t>FELIPE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11430</t>
+  </si>
+  <si>
+    <t>RAYANE ROBERTA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11463</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11408</t>
+  </si>
+  <si>
+    <t>FA-11352</t>
+  </si>
+  <si>
+    <t>ANDERSON QUEIROZ PINHEIRO</t>
+  </si>
+  <si>
+    <t>FA-11459</t>
+  </si>
+  <si>
+    <t>FA-11518</t>
+  </si>
+  <si>
+    <t>FA-11325</t>
+  </si>
+  <si>
+    <t>MAICON LOPES SILVA</t>
+  </si>
+  <si>
+    <t>FA-11265</t>
+  </si>
+  <si>
+    <t>ANNY KATARINA ACIOLE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11461</t>
+  </si>
+  <si>
+    <t>FA-11545</t>
+  </si>
+  <si>
+    <t>REGINALDO BENTO DA SILVA</t>
+  </si>
+  <si>
+    <t>JOÃO PAULO CONSÓRCIOS</t>
+  </si>
+  <si>
+    <t>FA-11348</t>
+  </si>
+  <si>
+    <t>FA-11347</t>
+  </si>
+  <si>
+    <t>FA-11446</t>
+  </si>
+  <si>
+    <t>FA-11362</t>
   </si>
   <si>
     <t>ANA CONCEIÇÃO CARNEIRO DE ALBUQUERQUE</t>
-  </si>
-  <si>
-    <t>VENCIDO ATÉ 30 DIAS</t>
-  </si>
-  <si>
-    <t>FA-11240</t>
-  </si>
-  <si>
-    <t>DIEGO TAYAO DANTAS</t>
-  </si>
-  <si>
-    <t>FATURA</t>
-  </si>
-  <si>
-    <t>FA-11155</t>
-  </si>
-  <si>
-    <t>OLIZIEL DA SILVA CARDOSO</t>
-  </si>
-  <si>
-    <t>FA-11496</t>
-  </si>
-  <si>
-    <t>ANDRE CAVALCANTI DA FE</t>
-  </si>
-  <si>
-    <t>AZ EMPREENDIMENTOS</t>
-  </si>
-  <si>
-    <t>FA-11447</t>
-  </si>
-  <si>
-    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
-  </si>
-  <si>
-    <t>FA-11421</t>
-  </si>
-  <si>
-    <t>FA-11406</t>
-  </si>
-  <si>
-    <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
-  </si>
-  <si>
-    <t>FA-11255</t>
-  </si>
-  <si>
-    <t>LEONARDO GOMES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11383</t>
-  </si>
-  <si>
-    <t>JOZILDO TARQUINO DE BRITO</t>
-  </si>
-  <si>
-    <t>FA-11419</t>
-  </si>
-  <si>
-    <t>YURI BATISTA DA COSTA</t>
-  </si>
-  <si>
-    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11189</t>
-  </si>
-  <si>
-    <t>FA-11182</t>
-  </si>
-  <si>
-    <t>MARCELO BENTO DE ARAUJO</t>
-  </si>
-  <si>
-    <t>FA-11069</t>
-  </si>
-  <si>
-    <t>ALBERTO MANOEL DOS REIS</t>
-  </si>
-  <si>
-    <t>PRIVADO</t>
-  </si>
-  <si>
-    <t>ND-11305</t>
-  </si>
-  <si>
-    <t>FA-11113</t>
-  </si>
-  <si>
-    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
-  </si>
-  <si>
-    <t>ND-10427</t>
-  </si>
-  <si>
-    <t>RICARDO ARAUJO DE MIRANDA</t>
-  </si>
-  <si>
-    <t>FA-11426</t>
-  </si>
-  <si>
-    <t>FA-11455</t>
-  </si>
-  <si>
-    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
-  </si>
-  <si>
-    <t>FA-11244</t>
-  </si>
-  <si>
-    <t>FA-11390</t>
-  </si>
-  <si>
-    <t>ADRIANO SANTOS DE CARVALHO</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
-  </si>
-  <si>
-    <t>FA-11115</t>
-  </si>
-  <si>
-    <t>FA-11256</t>
-  </si>
-  <si>
-    <t>FA-11407</t>
-  </si>
-  <si>
-    <t>FA-11424</t>
-  </si>
-  <si>
-    <t>FA-11183</t>
-  </si>
-  <si>
-    <t>FA-11361</t>
-  </si>
-  <si>
-    <t>RAMON TALLES BARBALHO DE FRANÇA</t>
-  </si>
-  <si>
-    <t>FA-11452</t>
-  </si>
-  <si>
-    <t>YAGO ELIAS COSTA BATISTA</t>
-  </si>
-  <si>
-    <t>FA-11346</t>
-  </si>
-  <si>
-    <t>FA-11114</t>
-  </si>
-  <si>
-    <t>FA-11456</t>
-  </si>
-  <si>
-    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11253</t>
-  </si>
-  <si>
-    <t>HOJE</t>
-  </si>
-  <si>
-    <t>FA-11387</t>
-  </si>
-  <si>
-    <t>A VENCER</t>
-  </si>
-  <si>
-    <t>FA-11147</t>
-  </si>
-  <si>
-    <t>FA-11516</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11392</t>
-  </si>
-  <si>
-    <t>FA-11458</t>
-  </si>
-  <si>
-    <t>FA-11153</t>
-  </si>
-  <si>
-    <t>FA-11462</t>
-  </si>
-  <si>
-    <t>FA-11517</t>
-  </si>
-  <si>
-    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11351</t>
-  </si>
-  <si>
-    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
-  </si>
-  <si>
-    <t>FA-11350</t>
-  </si>
-  <si>
-    <t>FA-11485</t>
-  </si>
-  <si>
-    <t>ROSSILY PEREIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11391</t>
-  </si>
-  <si>
-    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
-  </si>
-  <si>
-    <t>FA-11393</t>
-  </si>
-  <si>
-    <t>FA-11369</t>
-  </si>
-  <si>
-    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>FA-11460</t>
-  </si>
-  <si>
-    <t>FA-11500</t>
-  </si>
-  <si>
-    <t>WESCLY JEAN DE MEDEIROS</t>
-  </si>
-  <si>
-    <t>FA-11276</t>
-  </si>
-  <si>
-    <t>FELIPE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11111</t>
-  </si>
-  <si>
-    <t>FA-11497</t>
-  </si>
-  <si>
-    <t>FA-11430</t>
-  </si>
-  <si>
-    <t>RAYANE ROBERTA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11408</t>
-  </si>
-  <si>
-    <t>FA-11352</t>
-  </si>
-  <si>
-    <t>ANDERSON QUEIROZ PINHEIRO</t>
-  </si>
-  <si>
-    <t>FA-11459</t>
-  </si>
-  <si>
-    <t>FA-11518</t>
-  </si>
-  <si>
-    <t>FA-11463</t>
-  </si>
-  <si>
-    <t>LUCAS NAJA MOURA RODRIGUES</t>
-  </si>
-  <si>
-    <t>FA-11325</t>
-  </si>
-  <si>
-    <t>MAICON LOPES SILVA</t>
-  </si>
-  <si>
-    <t>FA-11265</t>
-  </si>
-  <si>
-    <t>ANNY KATARINA ACIOLE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11461</t>
-  </si>
-  <si>
-    <t>FA-11545</t>
-  </si>
-  <si>
-    <t>REGINALDO BENTO DA SILVA</t>
-  </si>
-  <si>
-    <t>JOÃO PAULO CONSÓRCIOS</t>
-  </si>
-  <si>
-    <t>FA-11348</t>
-  </si>
-  <si>
-    <t>FA-11347</t>
-  </si>
-  <si>
-    <t>FA-11446</t>
-  </si>
-  <si>
-    <t>FA-11362</t>
   </si>
 </sst>
 </file>
@@ -579,7 +573,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:S76"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.13657760620117" customWidth="1" style="1"/>
@@ -684,22 +678,22 @@
         <v>22</v>
       </c>
       <c r="B6" s="7">
-        <v>46030</v>
+        <v>46118</v>
       </c>
       <c r="C6" s="7">
-        <v>45992</v>
+        <v>46118</v>
       </c>
       <c r="D6" s="7">
-        <v>46030</v>
+        <v>46118</v>
       </c>
       <c r="E6" s="7">
-        <v>46044</v>
+        <v>46086</v>
       </c>
       <c r="F6" s="8">
-        <v>-106</v>
+        <v>-18</v>
       </c>
       <c r="G6" s="8">
-        <v>-106</v>
+        <v>-18</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>23</v>
@@ -717,7 +711,7 @@
         <v>26</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>27</v>
@@ -735,7 +729,7 @@
         <v>29</v>
       </c>
       <c r="S6" s="9">
-        <v>195.23</v>
+        <v>620</v>
       </c>
     </row>
     <row r="7" ht="23" customHeight="1">
@@ -743,37 +737,37 @@
         <v>22</v>
       </c>
       <c r="B7" s="7">
-        <v>46052</v>
+        <v>46125</v>
       </c>
       <c r="C7" s="7">
-        <v>45930</v>
+        <v>46104</v>
       </c>
       <c r="D7" s="7">
-        <v>46052</v>
+        <v>46104</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F7" s="8">
-        <v>-84</v>
+        <v>-32</v>
       </c>
       <c r="G7" s="8">
-        <v>-84</v>
+        <v>-11</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>30</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M7" s="6" t="s">
         <v>25</v>
@@ -791,10 +785,10 @@
         <v>25</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="S7" s="9">
-        <v>185.5</v>
+        <v>165.25</v>
       </c>
     </row>
     <row r="8" ht="23" customHeight="1">
@@ -802,28 +796,28 @@
         <v>22</v>
       </c>
       <c r="B8" s="7">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="C8" s="7">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="D8" s="7">
-        <v>46118</v>
+        <v>46125</v>
       </c>
       <c r="E8" s="7">
-        <v>46086</v>
+        <v>46122</v>
       </c>
       <c r="F8" s="8">
-        <v>-18</v>
+        <v>-11</v>
       </c>
       <c r="G8" s="8">
-        <v>-18</v>
+        <v>-11</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>33</v>
@@ -835,7 +829,7 @@
         <v>34</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>27</v>
@@ -847,13 +841,13 @@
         <v>25</v>
       </c>
       <c r="Q8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R8" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R8" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="S8" s="9">
-        <v>620</v>
+        <v>650</v>
       </c>
     </row>
     <row r="9" ht="23" customHeight="1">
@@ -864,25 +858,25 @@
         <v>46125</v>
       </c>
       <c r="C9" s="7">
-        <v>46104</v>
+        <v>46125</v>
       </c>
       <c r="D9" s="7">
-        <v>46104</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>25</v>
+        <v>46125</v>
+      </c>
+      <c r="E9" s="7">
+        <v>46119</v>
       </c>
       <c r="F9" s="8">
-        <v>-32</v>
+        <v>-11</v>
       </c>
       <c r="G9" s="8">
         <v>-11</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>36</v>
@@ -894,7 +888,7 @@
         <v>37</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>27</v>
@@ -906,13 +900,13 @@
         <v>25</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S9" s="9">
-        <v>165.25</v>
+        <v>650</v>
       </c>
     </row>
     <row r="10" ht="23" customHeight="1">
@@ -929,7 +923,7 @@
         <v>46125</v>
       </c>
       <c r="E10" s="7">
-        <v>46122</v>
+        <v>46118</v>
       </c>
       <c r="F10" s="8">
         <v>-11</v>
@@ -938,10 +932,10 @@
         <v>-11</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>38</v>
@@ -950,7 +944,7 @@
         <v>25</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="M10" s="6" t="s">
         <v>25</v>
@@ -965,13 +959,13 @@
         <v>25</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S10" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="11" ht="23" customHeight="1">
@@ -988,7 +982,7 @@
         <v>46125</v>
       </c>
       <c r="E11" s="7">
-        <v>46119</v>
+        <v>46087</v>
       </c>
       <c r="F11" s="8">
         <v>-11</v>
@@ -997,22 +991,22 @@
         <v>-11</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N11" s="6" t="s">
         <v>27</v>
@@ -1024,13 +1018,13 @@
         <v>25</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R11" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S11" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="12" ht="23" customHeight="1">
@@ -1047,7 +1041,7 @@
         <v>46125</v>
       </c>
       <c r="E12" s="7">
-        <v>46118</v>
+        <v>46113</v>
       </c>
       <c r="F12" s="8">
         <v>-11</v>
@@ -1056,22 +1050,22 @@
         <v>-11</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="N12" s="6" t="s">
         <v>27</v>
@@ -1083,7 +1077,7 @@
         <v>25</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>29</v>
@@ -1097,40 +1091,40 @@
         <v>22</v>
       </c>
       <c r="B13" s="7">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="C13" s="7">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="D13" s="7">
-        <v>46125</v>
-      </c>
-      <c r="E13" s="7">
-        <v>46113</v>
+        <v>46118</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F13" s="8">
-        <v>-11</v>
+        <v>-18</v>
       </c>
       <c r="G13" s="8">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>45</v>
-      </c>
       <c r="M13" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>27</v>
@@ -1142,13 +1136,13 @@
         <v>25</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R13" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S13" s="9">
-        <v>680</v>
+        <v>130.16</v>
       </c>
     </row>
     <row r="14" ht="23" customHeight="1">
@@ -1156,38 +1150,38 @@
         <v>22</v>
       </c>
       <c r="B14" s="7">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="C14" s="7">
-        <v>46125</v>
+        <v>46118</v>
       </c>
       <c r="D14" s="7">
-        <v>46125</v>
-      </c>
-      <c r="E14" s="7">
-        <v>46087</v>
+        <v>46118</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F14" s="8">
-        <v>-11</v>
+        <v>-18</v>
       </c>
       <c r="G14" s="8">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>47</v>
-      </c>
       <c r="M14" s="6" t="s">
         <v>25</v>
       </c>
@@ -1201,13 +1195,13 @@
         <v>25</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R14" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S14" s="9">
-        <v>680</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" ht="23" customHeight="1">
@@ -1215,7 +1209,7 @@
         <v>22</v>
       </c>
       <c r="B15" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="C15" s="7">
         <v>46118</v>
@@ -1230,25 +1224,25 @@
         <v>-18</v>
       </c>
       <c r="G15" s="8">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="N15" s="6" t="s">
         <v>27</v>
@@ -1266,7 +1260,7 @@
         <v>29</v>
       </c>
       <c r="S15" s="9">
-        <v>130.16</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" ht="23" customHeight="1">
@@ -1274,40 +1268,40 @@
         <v>22</v>
       </c>
       <c r="B16" s="7">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="C16" s="7">
-        <v>46118</v>
+        <v>46111</v>
       </c>
       <c r="D16" s="7">
-        <v>46118</v>
+        <v>46111</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F16" s="8">
-        <v>-18</v>
+        <v>-25</v>
       </c>
       <c r="G16" s="8">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>27</v>
@@ -1325,7 +1319,7 @@
         <v>29</v>
       </c>
       <c r="S16" s="9">
-        <v>400</v>
+        <v>119.57</v>
       </c>
     </row>
     <row r="17" ht="23" customHeight="1">
@@ -1333,37 +1327,37 @@
         <v>22</v>
       </c>
       <c r="B17" s="7">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="C17" s="7">
-        <v>46118</v>
+        <v>46104</v>
       </c>
       <c r="D17" s="7">
-        <v>46118</v>
+        <v>46104</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F17" s="8">
-        <v>-18</v>
+        <v>-32</v>
       </c>
       <c r="G17" s="8">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>25</v>
@@ -1381,10 +1375,10 @@
         <v>25</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S17" s="9">
-        <v>260</v>
+        <v>357.49</v>
       </c>
     </row>
     <row r="18" ht="23" customHeight="1">
@@ -1392,50 +1386,50 @@
         <v>22</v>
       </c>
       <c r="B18" s="7">
-        <v>46128</v>
+        <v>46132</v>
       </c>
       <c r="C18" s="7">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="D18" s="7">
-        <v>46111</v>
+        <v>46118</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F18" s="8">
-        <v>-25</v>
+        <v>-18</v>
       </c>
       <c r="G18" s="8">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J18" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="K18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O18" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="Q18" s="6" t="s">
         <v>25</v>
       </c>
@@ -1443,7 +1437,7 @@
         <v>29</v>
       </c>
       <c r="S18" s="9">
-        <v>119.57</v>
+        <v>91.54</v>
       </c>
     </row>
     <row r="19" ht="23" customHeight="1">
@@ -1451,28 +1445,28 @@
         <v>22</v>
       </c>
       <c r="B19" s="7">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="C19" s="7">
-        <v>46104</v>
+        <v>46082</v>
       </c>
       <c r="D19" s="7">
-        <v>46104</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E19" s="7">
+        <v>46097</v>
       </c>
       <c r="F19" s="8">
-        <v>-32</v>
+        <v>-4</v>
       </c>
       <c r="G19" s="8">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>54</v>
@@ -1481,28 +1475,28 @@
         <v>25</v>
       </c>
       <c r="L19" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="M19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O19" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="P19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q19" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="R19" s="6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="S19" s="9">
-        <v>357.49</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="20" ht="23" customHeight="1">
@@ -1528,10 +1522,10 @@
         <v>-4</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>56</v>
@@ -1552,7 +1546,7 @@
         <v>27</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="Q20" s="6" t="s">
         <v>25</v>
@@ -1561,7 +1555,7 @@
         <v>29</v>
       </c>
       <c r="S20" s="9">
-        <v>91.54</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21" ht="23" customHeight="1">
@@ -1572,25 +1566,25 @@
         <v>46132</v>
       </c>
       <c r="C21" s="7">
-        <v>46082</v>
+        <v>45901</v>
       </c>
       <c r="D21" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E21" s="7">
-        <v>46097</v>
+        <v>45938</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F21" s="8">
-        <v>-4</v>
+        <v>-198</v>
       </c>
       <c r="G21" s="8">
         <v>-4</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>59</v>
@@ -1599,7 +1593,7 @@
         <v>25</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M21" s="6" t="s">
         <v>25</v>
@@ -1614,13 +1608,13 @@
         <v>25</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S21" s="9">
-        <v>146.55</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" ht="23" customHeight="1">
@@ -1631,37 +1625,37 @@
         <v>46132</v>
       </c>
       <c r="C22" s="7">
-        <v>46118</v>
+        <v>46132</v>
       </c>
       <c r="D22" s="7">
-        <v>46118</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E22" s="7">
+        <v>46119</v>
       </c>
       <c r="F22" s="8">
-        <v>-18</v>
+        <v>-4</v>
       </c>
       <c r="G22" s="8">
         <v>-4</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K22" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="N22" s="6" t="s">
         <v>27</v>
@@ -1673,13 +1667,13 @@
         <v>25</v>
       </c>
       <c r="Q22" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R22" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S22" s="9">
-        <v>200</v>
+        <v>620</v>
       </c>
     </row>
     <row r="23" ht="23" customHeight="1">
@@ -1690,16 +1684,16 @@
         <v>46132</v>
       </c>
       <c r="C23" s="7">
-        <v>45901</v>
+        <v>46132</v>
       </c>
       <c r="D23" s="7">
-        <v>45938</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>25</v>
+        <v>46132</v>
+      </c>
+      <c r="E23" s="7">
+        <v>46118</v>
       </c>
       <c r="F23" s="8">
-        <v>-198</v>
+        <v>-4</v>
       </c>
       <c r="G23" s="8">
         <v>-4</v>
@@ -1708,16 +1702,16 @@
         <v>23</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="M23" s="6" t="s">
         <v>25</v>
@@ -1732,13 +1726,13 @@
         <v>25</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R23" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S23" s="9">
-        <v>546</v>
+        <v>620</v>
       </c>
     </row>
     <row r="24" ht="23" customHeight="1">
@@ -1755,7 +1749,7 @@
         <v>46132</v>
       </c>
       <c r="E24" s="7">
-        <v>46118</v>
+        <v>46086</v>
       </c>
       <c r="F24" s="8">
         <v>-4</v>
@@ -1764,10 +1758,10 @@
         <v>-4</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>64</v>
@@ -1776,10 +1770,10 @@
         <v>25</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
         <v>27</v>
@@ -1791,7 +1785,7 @@
         <v>25</v>
       </c>
       <c r="Q24" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R24" s="6" t="s">
         <v>29</v>
@@ -1814,7 +1808,7 @@
         <v>46132</v>
       </c>
       <c r="E25" s="7">
-        <v>46119</v>
+        <v>46112</v>
       </c>
       <c r="F25" s="8">
         <v>-4</v>
@@ -1823,10 +1817,10 @@
         <v>-4</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>65</v>
@@ -1838,7 +1832,7 @@
         <v>66</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="N25" s="6" t="s">
         <v>27</v>
@@ -1850,13 +1844,13 @@
         <v>25</v>
       </c>
       <c r="Q25" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S25" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="26" ht="23" customHeight="1">
@@ -1873,7 +1867,7 @@
         <v>46132</v>
       </c>
       <c r="E26" s="7">
-        <v>46086</v>
+        <v>46119</v>
       </c>
       <c r="F26" s="8">
         <v>-4</v>
@@ -1882,10 +1876,10 @@
         <v>-4</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>67</v>
@@ -1894,10 +1888,10 @@
         <v>25</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N26" s="6" t="s">
         <v>27</v>
@@ -1909,13 +1903,13 @@
         <v>25</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R26" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S26" s="9">
-        <v>620</v>
+        <v>650</v>
       </c>
     </row>
     <row r="27" ht="23" customHeight="1">
@@ -1932,7 +1926,7 @@
         <v>46132</v>
       </c>
       <c r="E27" s="7">
-        <v>46112</v>
+        <v>46057</v>
       </c>
       <c r="F27" s="8">
         <v>-4</v>
@@ -1941,10 +1935,10 @@
         <v>-4</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>68</v>
@@ -1953,7 +1947,7 @@
         <v>25</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>25</v>
@@ -1968,13 +1962,13 @@
         <v>25</v>
       </c>
       <c r="Q27" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R27" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S27" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="28" ht="23" customHeight="1">
@@ -1991,7 +1985,7 @@
         <v>46132</v>
       </c>
       <c r="E28" s="7">
-        <v>46119</v>
+        <v>46087</v>
       </c>
       <c r="F28" s="8">
         <v>-4</v>
@@ -2000,22 +1994,22 @@
         <v>-4</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N28" s="6" t="s">
         <v>27</v>
@@ -2027,13 +2021,13 @@
         <v>25</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R28" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S28" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="29" ht="23" customHeight="1">
@@ -2050,7 +2044,7 @@
         <v>46132</v>
       </c>
       <c r="E29" s="7">
-        <v>46057</v>
+        <v>46118</v>
       </c>
       <c r="F29" s="8">
         <v>-4</v>
@@ -2059,20 +2053,20 @@
         <v>-4</v>
       </c>
       <c r="H29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I29" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="M29" s="6" t="s">
         <v>25</v>
       </c>
@@ -2086,13 +2080,13 @@
         <v>25</v>
       </c>
       <c r="Q29" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R29" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S29" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="30" ht="23" customHeight="1">
@@ -2109,7 +2103,7 @@
         <v>46132</v>
       </c>
       <c r="E30" s="7">
-        <v>46087</v>
+        <v>46113</v>
       </c>
       <c r="F30" s="8">
         <v>-4</v>
@@ -2118,22 +2112,22 @@
         <v>-4</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K30" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="N30" s="6" t="s">
         <v>27</v>
@@ -2145,7 +2139,7 @@
         <v>25</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R30" s="6" t="s">
         <v>29</v>
@@ -2159,40 +2153,40 @@
         <v>22</v>
       </c>
       <c r="B31" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="C31" s="7">
-        <v>46132</v>
+        <v>46118</v>
       </c>
       <c r="D31" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E31" s="7">
-        <v>46113</v>
+        <v>46111</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F31" s="8">
-        <v>-4</v>
+        <v>-25</v>
       </c>
       <c r="G31" s="8">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="M31" s="6" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="N31" s="6" t="s">
         <v>27</v>
@@ -2204,13 +2198,13 @@
         <v>25</v>
       </c>
       <c r="Q31" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="R31" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R31" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="S31" s="9">
-        <v>680</v>
+        <v>321.17</v>
       </c>
     </row>
     <row r="32" ht="23" customHeight="1">
@@ -2218,38 +2212,38 @@
         <v>22</v>
       </c>
       <c r="B32" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="C32" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="D32" s="7">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="E32" s="7">
-        <v>46118</v>
+        <v>46100</v>
       </c>
       <c r="F32" s="8">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="G32" s="8">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J32" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L32" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="K32" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>37</v>
-      </c>
       <c r="M32" s="6" t="s">
         <v>25</v>
       </c>
@@ -2263,10 +2257,10 @@
         <v>25</v>
       </c>
       <c r="Q32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R32" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="R32" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="S32" s="9">
         <v>680</v>
@@ -2277,37 +2271,37 @@
         <v>22</v>
       </c>
       <c r="B33" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="C33" s="7">
-        <v>46118</v>
+        <v>46082</v>
       </c>
       <c r="D33" s="7">
-        <v>46111</v>
+        <v>46125</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F33" s="8">
-        <v>-25</v>
+        <v>-11</v>
       </c>
       <c r="G33" s="8">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="K33" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>25</v>
@@ -2325,10 +2319,10 @@
         <v>25</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="S33" s="9">
-        <v>321.17</v>
+        <v>79.05</v>
       </c>
     </row>
     <row r="34" ht="23" customHeight="1">
@@ -2336,40 +2330,40 @@
         <v>22</v>
       </c>
       <c r="B34" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="C34" s="7">
-        <v>46133</v>
+        <v>46132</v>
       </c>
       <c r="D34" s="7">
-        <v>46133</v>
-      </c>
-      <c r="E34" s="7">
-        <v>46100</v>
+        <v>46132</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F34" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G34" s="8">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J34" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L34" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="K34" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="M34" s="6" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>27</v>
@@ -2381,13 +2375,13 @@
         <v>25</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S34" s="9">
-        <v>680</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
@@ -2398,34 +2392,34 @@
         <v>46134</v>
       </c>
       <c r="C35" s="7">
-        <v>46082</v>
+        <v>46132</v>
       </c>
       <c r="D35" s="7">
-        <v>46125</v>
+        <v>46132</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F35" s="8">
-        <v>-11</v>
+        <v>-4</v>
       </c>
       <c r="G35" s="8">
         <v>-2</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>25</v>
@@ -2443,10 +2437,10 @@
         <v>25</v>
       </c>
       <c r="R35" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S35" s="9">
-        <v>79.05</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
@@ -2454,28 +2448,28 @@
         <v>22</v>
       </c>
       <c r="B36" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="C36" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="D36" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F36" s="8">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="G36" s="8">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J36" s="6" t="s">
         <v>78</v>
@@ -2484,10 +2478,10 @@
         <v>25</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="N36" s="6" t="s">
         <v>27</v>
@@ -2505,7 +2499,7 @@
         <v>29</v>
       </c>
       <c r="S36" s="9">
-        <v>200</v>
+        <v>550</v>
       </c>
     </row>
     <row r="37" ht="23" customHeight="1">
@@ -2513,7 +2507,7 @@
         <v>22</v>
       </c>
       <c r="B37" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="C37" s="7">
         <v>46132</v>
@@ -2528,23 +2522,23 @@
         <v>-4</v>
       </c>
       <c r="G37" s="8">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="J37" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L37" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="K37" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="M37" s="6" t="s">
         <v>25</v>
       </c>
@@ -2555,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="P37" s="6" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>25</v>
@@ -2564,7 +2558,7 @@
         <v>29</v>
       </c>
       <c r="S37" s="9">
-        <v>200</v>
+        <v>650</v>
       </c>
     </row>
     <row r="38" ht="23" customHeight="1">
@@ -2572,28 +2566,28 @@
         <v>22</v>
       </c>
       <c r="B38" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="C38" s="7">
-        <v>46125</v>
+        <v>46111</v>
       </c>
       <c r="D38" s="7">
-        <v>46125</v>
+        <v>46111</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F38" s="8">
-        <v>-11</v>
+        <v>-25</v>
       </c>
       <c r="G38" s="8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>81</v>
@@ -2602,7 +2596,7 @@
         <v>25</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>25</v>
@@ -2611,7 +2605,7 @@
         <v>27</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>25</v>
@@ -2623,7 +2617,7 @@
         <v>29</v>
       </c>
       <c r="S38" s="9">
-        <v>550</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" ht="23" customHeight="1">
@@ -2631,49 +2625,49 @@
         <v>22</v>
       </c>
       <c r="B39" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="C39" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="D39" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F39" s="8">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="G39" s="8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J39" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O39" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K39" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="M39" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N39" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O39" s="6" t="s">
-        <v>27</v>
-      </c>
       <c r="P39" s="6" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="Q39" s="6" t="s">
         <v>25</v>
@@ -2682,7 +2676,7 @@
         <v>29</v>
       </c>
       <c r="S39" s="9">
-        <v>650</v>
+        <v>302.72</v>
       </c>
     </row>
     <row r="40" ht="23" customHeight="1">
@@ -2690,58 +2684,58 @@
         <v>22</v>
       </c>
       <c r="B40" s="7">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="C40" s="7">
-        <v>46111</v>
+        <v>46082</v>
       </c>
       <c r="D40" s="7">
-        <v>46111</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>25</v>
+        <v>46139</v>
+      </c>
+      <c r="E40" s="7">
+        <v>46097</v>
       </c>
       <c r="F40" s="8">
-        <v>-25</v>
+        <v>3</v>
       </c>
       <c r="G40" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S40" s="9">
-        <v>180</v>
+        <v>146.55</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1">
@@ -2749,37 +2743,37 @@
         <v>22</v>
       </c>
       <c r="B41" s="7">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="C41" s="7">
-        <v>46125</v>
+        <v>46111</v>
       </c>
       <c r="D41" s="7">
-        <v>46125</v>
+        <v>46083</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F41" s="8">
-        <v>-11</v>
+        <v>-53</v>
       </c>
       <c r="G41" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I41" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K41" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>25</v>
@@ -2788,7 +2782,7 @@
         <v>27</v>
       </c>
       <c r="O41" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P41" s="6" t="s">
         <v>25</v>
@@ -2800,7 +2794,7 @@
         <v>29</v>
       </c>
       <c r="S41" s="9">
-        <v>302.72</v>
+        <v>320</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1">
@@ -2811,13 +2805,13 @@
         <v>46139</v>
       </c>
       <c r="C42" s="7">
-        <v>46082</v>
+        <v>46139</v>
       </c>
       <c r="D42" s="7">
         <v>46139</v>
       </c>
       <c r="E42" s="7">
-        <v>46097</v>
+        <v>46119</v>
       </c>
       <c r="F42" s="8">
         <v>3</v>
@@ -2832,22 +2826,22 @@
         <v>25</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="K42" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>25</v>
@@ -2856,10 +2850,10 @@
         <v>28</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S42" s="9">
-        <v>146.55</v>
+        <v>600</v>
       </c>
     </row>
     <row r="43" ht="23" customHeight="1">
@@ -2870,55 +2864,55 @@
         <v>46139</v>
       </c>
       <c r="C43" s="7">
-        <v>46111</v>
+        <v>46139</v>
       </c>
       <c r="D43" s="7">
-        <v>46083</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>25</v>
+        <v>46139</v>
+      </c>
+      <c r="E43" s="7">
+        <v>46112</v>
       </c>
       <c r="F43" s="8">
-        <v>-53</v>
+        <v>3</v>
       </c>
       <c r="G43" s="8">
         <v>3</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I43" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K43" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P43" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q43" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R43" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S43" s="9">
-        <v>320</v>
+        <v>600</v>
       </c>
     </row>
     <row r="44" ht="23" customHeight="1">
@@ -2950,28 +2944,28 @@
         <v>25</v>
       </c>
       <c r="J44" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L44" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="K44" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="M44" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R44" s="6" t="s">
         <v>29</v>
@@ -2994,7 +2988,7 @@
         <v>46139</v>
       </c>
       <c r="E45" s="7">
-        <v>46112</v>
+        <v>46119</v>
       </c>
       <c r="F45" s="8">
         <v>3</v>
@@ -3009,34 +3003,34 @@
         <v>25</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O45" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P45" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R45" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R45" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="S45" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="46" ht="23" customHeight="1">
@@ -3050,52 +3044,52 @@
         <v>46139</v>
       </c>
       <c r="D46" s="7">
-        <v>46139</v>
+        <v>46104</v>
       </c>
       <c r="E46" s="7">
-        <v>46119</v>
+        <v>46057</v>
       </c>
       <c r="F46" s="8">
-        <v>3</v>
+        <v>-32</v>
       </c>
       <c r="G46" s="8">
         <v>3</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I46" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q46" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R46" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S46" s="9">
-        <v>600</v>
+        <v>620</v>
       </c>
     </row>
     <row r="47" ht="23" customHeight="1">
@@ -3109,52 +3103,52 @@
         <v>46139</v>
       </c>
       <c r="D47" s="7">
-        <v>46104</v>
+        <v>46139</v>
       </c>
       <c r="E47" s="7">
-        <v>46057</v>
+        <v>46112</v>
       </c>
       <c r="F47" s="8">
-        <v>-32</v>
+        <v>3</v>
       </c>
       <c r="G47" s="8">
         <v>3</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="M47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P47" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q47" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R47" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S47" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="48" ht="23" customHeight="1">
@@ -3171,7 +3165,7 @@
         <v>46139</v>
       </c>
       <c r="E48" s="7">
-        <v>46119</v>
+        <v>46100</v>
       </c>
       <c r="F48" s="8">
         <v>3</v>
@@ -3186,34 +3180,34 @@
         <v>25</v>
       </c>
       <c r="J48" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L48" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="K48" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L48" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="M48" s="6" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q48" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R48" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S48" s="9">
-        <v>620</v>
+        <v>630</v>
       </c>
     </row>
     <row r="49" ht="23" customHeight="1">
@@ -3230,7 +3224,7 @@
         <v>46139</v>
       </c>
       <c r="E49" s="7">
-        <v>46127</v>
+        <v>46100</v>
       </c>
       <c r="F49" s="8">
         <v>3</v>
@@ -3251,22 +3245,22 @@
         <v>25</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P49" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q49" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R49" s="6" t="s">
         <v>29</v>
@@ -3289,7 +3283,7 @@
         <v>46139</v>
       </c>
       <c r="E50" s="7">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="F50" s="8">
         <v>3</v>
@@ -3304,28 +3298,28 @@
         <v>25</v>
       </c>
       <c r="J50" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L50" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="K50" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="M50" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q50" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R50" s="6" t="s">
         <v>29</v>
@@ -3348,7 +3342,7 @@
         <v>46139</v>
       </c>
       <c r="E51" s="7">
-        <v>46100</v>
+        <v>46119</v>
       </c>
       <c r="F51" s="8">
         <v>3</v>
@@ -3363,28 +3357,28 @@
         <v>25</v>
       </c>
       <c r="J51" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L51" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="K51" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="M51" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P51" s="6" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="Q51" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R51" s="6" t="s">
         <v>29</v>
@@ -3407,7 +3401,7 @@
         <v>46139</v>
       </c>
       <c r="E52" s="7">
-        <v>46119</v>
+        <v>46127</v>
       </c>
       <c r="F52" s="8">
         <v>3</v>
@@ -3434,16 +3428,16 @@
         <v>25</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="Q52" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R52" s="6" t="s">
         <v>29</v>
@@ -3466,7 +3460,7 @@
         <v>46139</v>
       </c>
       <c r="E53" s="7">
-        <v>46112</v>
+        <v>46127</v>
       </c>
       <c r="F53" s="8">
         <v>3</v>
@@ -3493,22 +3487,22 @@
         <v>25</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O53" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P53" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q53" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R53" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S53" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="54" ht="23" customHeight="1">
@@ -3522,19 +3516,19 @@
         <v>46139</v>
       </c>
       <c r="D54" s="7">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="E54" s="7">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="F54" s="8">
-        <v>3</v>
+        <v>-4</v>
       </c>
       <c r="G54" s="8">
         <v>3</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I54" s="6" t="s">
         <v>25</v>
@@ -3546,28 +3540,28 @@
         <v>25</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q54" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R54" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R54" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="S54" s="9">
-        <v>630</v>
+        <v>650</v>
       </c>
     </row>
     <row r="55" ht="23" customHeight="1">
@@ -3584,7 +3578,7 @@
         <v>46139</v>
       </c>
       <c r="E55" s="7">
-        <v>46101</v>
+        <v>46119</v>
       </c>
       <c r="F55" s="8">
         <v>3</v>
@@ -3605,22 +3599,22 @@
         <v>25</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q55" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R55" s="6" t="s">
         <v>29</v>
@@ -3643,7 +3637,7 @@
         <v>46139</v>
       </c>
       <c r="E56" s="7">
-        <v>46119</v>
+        <v>46101</v>
       </c>
       <c r="F56" s="8">
         <v>3</v>
@@ -3658,28 +3652,28 @@
         <v>25</v>
       </c>
       <c r="J56" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L56" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="K56" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="M56" s="6" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q56" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R56" s="6" t="s">
         <v>29</v>
@@ -3699,19 +3693,19 @@
         <v>46139</v>
       </c>
       <c r="D57" s="7">
-        <v>46139</v>
+        <v>46104</v>
       </c>
       <c r="E57" s="7">
-        <v>46127</v>
+        <v>46057</v>
       </c>
       <c r="F57" s="8">
-        <v>3</v>
+        <v>-32</v>
       </c>
       <c r="G57" s="8">
         <v>3</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I57" s="6" t="s">
         <v>25</v>
@@ -3723,22 +3717,22 @@
         <v>25</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="M57" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P57" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q57" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R57" s="6" t="s">
         <v>29</v>
@@ -3776,28 +3770,28 @@
         <v>25</v>
       </c>
       <c r="J58" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L58" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="K58" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L58" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="M58" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q58" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R58" s="6" t="s">
         <v>29</v>
@@ -3817,52 +3811,52 @@
         <v>46139</v>
       </c>
       <c r="D59" s="7">
-        <v>46104</v>
+        <v>46139</v>
       </c>
       <c r="E59" s="7">
-        <v>46057</v>
+        <v>46119</v>
       </c>
       <c r="F59" s="8">
-        <v>-32</v>
+        <v>3</v>
       </c>
       <c r="G59" s="8">
         <v>3</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J59" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L59" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="K59" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L59" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="M59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P59" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q59" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R59" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S59" s="9">
-        <v>650</v>
+        <v>670</v>
       </c>
     </row>
     <row r="60" ht="23" customHeight="1">
@@ -3876,19 +3870,19 @@
         <v>46139</v>
       </c>
       <c r="D60" s="7">
-        <v>46132</v>
+        <v>46139</v>
       </c>
       <c r="E60" s="7">
-        <v>46122</v>
+        <v>46119</v>
       </c>
       <c r="F60" s="8">
-        <v>-4</v>
+        <v>3</v>
       </c>
       <c r="G60" s="8">
         <v>3</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I60" s="6" t="s">
         <v>25</v>
@@ -3900,28 +3894,28 @@
         <v>25</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>39</v>
+        <v>114</v>
       </c>
       <c r="M60" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q60" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R60" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S60" s="9">
-        <v>650</v>
+        <v>680</v>
       </c>
     </row>
     <row r="61" ht="23" customHeight="1">
@@ -3938,7 +3932,7 @@
         <v>46139</v>
       </c>
       <c r="E61" s="7">
-        <v>46119</v>
+        <v>46113</v>
       </c>
       <c r="F61" s="8">
         <v>3</v>
@@ -3953,34 +3947,34 @@
         <v>25</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K61" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>115</v>
+        <v>42</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O61" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P61" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q61" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R61" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S61" s="9">
-        <v>670</v>
+        <v>680</v>
       </c>
     </row>
     <row r="62" ht="23" customHeight="1">
@@ -3997,7 +3991,7 @@
         <v>46139</v>
       </c>
       <c r="E62" s="7">
-        <v>46113</v>
+        <v>46100</v>
       </c>
       <c r="F62" s="8">
         <v>3</v>
@@ -4018,22 +4012,22 @@
         <v>25</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>45</v>
+        <v>117</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q62" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R62" s="6" t="s">
         <v>29</v>
@@ -4056,7 +4050,7 @@
         <v>46139</v>
       </c>
       <c r="E63" s="7">
-        <v>46100</v>
+        <v>46119</v>
       </c>
       <c r="F63" s="8">
         <v>3</v>
@@ -4071,31 +4065,31 @@
         <v>25</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K63" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="M63" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O63" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P63" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R63" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="R63" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="S63" s="9">
         <v>680</v>
@@ -4115,7 +4109,7 @@
         <v>46139</v>
       </c>
       <c r="E64" s="7">
-        <v>46119</v>
+        <v>46127</v>
       </c>
       <c r="F64" s="8">
         <v>3</v>
@@ -4136,25 +4130,25 @@
         <v>25</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M64" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="Q64" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R64" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S64" s="9">
         <v>680</v>
@@ -4174,7 +4168,7 @@
         <v>46139</v>
       </c>
       <c r="E65" s="7">
-        <v>46127</v>
+        <v>46099</v>
       </c>
       <c r="F65" s="8">
         <v>3</v>
@@ -4195,28 +4189,28 @@
         <v>25</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>57</v>
+        <v>121</v>
       </c>
       <c r="M65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P65" s="6" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="Q65" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R65" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="R65" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="S65" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="66" ht="23" customHeight="1">
@@ -4233,7 +4227,7 @@
         <v>46139</v>
       </c>
       <c r="E66" s="7">
-        <v>46119</v>
+        <v>46092</v>
       </c>
       <c r="F66" s="8">
         <v>3</v>
@@ -4248,34 +4242,34 @@
         <v>25</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q66" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R66" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S66" s="9">
-        <v>680</v>
+        <v>700</v>
       </c>
     </row>
     <row r="67" ht="23" customHeight="1">
@@ -4292,7 +4286,7 @@
         <v>46139</v>
       </c>
       <c r="E67" s="7">
-        <v>46099</v>
+        <v>46119</v>
       </c>
       <c r="F67" s="8">
         <v>3</v>
@@ -4307,31 +4301,31 @@
         <v>25</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K67" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="M67" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P67" s="6" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="Q67" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R67" s="6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="S67" s="9">
         <v>700</v>
@@ -4351,7 +4345,7 @@
         <v>46139</v>
       </c>
       <c r="E68" s="7">
-        <v>46092</v>
+        <v>46129</v>
       </c>
       <c r="F68" s="8">
         <v>3</v>
@@ -4378,22 +4372,22 @@
         <v>25</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q68" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>29</v>
+        <v>127</v>
       </c>
       <c r="S68" s="9">
-        <v>700</v>
+        <v>800</v>
       </c>
     </row>
     <row r="69" ht="23" customHeight="1">
@@ -4401,58 +4395,58 @@
         <v>22</v>
       </c>
       <c r="B69" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C69" s="7">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="D69" s="7">
-        <v>46139</v>
-      </c>
-      <c r="E69" s="7">
-        <v>46119</v>
+        <v>46132</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F69" s="8">
-        <v>3</v>
+        <v>-4</v>
       </c>
       <c r="G69" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="O69" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P69" s="6" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="Q69" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R69" s="6" t="s">
         <v>29</v>
       </c>
       <c r="S69" s="9">
-        <v>700</v>
+        <v>110.69</v>
       </c>
     </row>
     <row r="70" ht="23" customHeight="1">
@@ -4460,58 +4454,58 @@
         <v>22</v>
       </c>
       <c r="B70" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="C70" s="7">
-        <v>46139</v>
+        <v>46132</v>
       </c>
       <c r="D70" s="7">
-        <v>46139</v>
-      </c>
-      <c r="E70" s="7">
-        <v>46129</v>
+        <v>46132</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="F70" s="8">
-        <v>3</v>
+        <v>-4</v>
       </c>
       <c r="G70" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="M70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q70" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R70" s="6" t="s">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="S70" s="9">
-        <v>800</v>
+        <v>124.25</v>
       </c>
     </row>
     <row r="71" ht="23" customHeight="1">
@@ -4522,34 +4516,34 @@
         <v>46140</v>
       </c>
       <c r="C71" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="D71" s="7">
-        <v>46132</v>
+        <v>46125</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F71" s="8">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="G71" s="8">
         <v>4</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I71" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K71" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="M71" s="6" t="s">
         <v>25</v>
@@ -4558,7 +4552,7 @@
         <v>27</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P71" s="6" t="s">
         <v>25</v>
@@ -4567,10 +4561,10 @@
         <v>25</v>
       </c>
       <c r="R71" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S71" s="9">
-        <v>110.69</v>
+        <v>408.24</v>
       </c>
     </row>
     <row r="72" ht="23" customHeight="1">
@@ -4581,55 +4575,55 @@
         <v>46140</v>
       </c>
       <c r="C72" s="7">
-        <v>46132</v>
+        <v>46140</v>
       </c>
       <c r="D72" s="7">
-        <v>46132</v>
-      </c>
-      <c r="E72" s="7" t="s">
-        <v>25</v>
+        <v>46140</v>
+      </c>
+      <c r="E72" s="7">
+        <v>46100</v>
       </c>
       <c r="F72" s="8">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="G72" s="8">
         <v>4</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I72" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K72" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="M72" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>25</v>
       </c>
       <c r="Q72" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="R72" s="6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="S72" s="9">
-        <v>124.25</v>
+        <v>680</v>
       </c>
     </row>
     <row r="73" ht="23" customHeight="1">
@@ -4637,46 +4631,46 @@
         <v>22</v>
       </c>
       <c r="B73" s="7">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="C73" s="7">
-        <v>46125</v>
+        <v>45930</v>
       </c>
       <c r="D73" s="7">
-        <v>46125</v>
+        <v>46142</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>25</v>
       </c>
       <c r="F73" s="8">
-        <v>-11</v>
+        <v>6</v>
       </c>
       <c r="G73" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I73" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="K73" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>55</v>
+        <v>132</v>
       </c>
       <c r="M73" s="6" t="s">
         <v>25</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="O73" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P73" s="6" t="s">
         <v>25</v>
@@ -4685,187 +4679,69 @@
         <v>25</v>
       </c>
       <c r="R73" s="6" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="S73" s="9">
-        <v>408.24</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="74" ht="23" customHeight="1">
-      <c r="A74" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B74" s="7">
-        <v>46140</v>
-      </c>
-      <c r="C74" s="7">
-        <v>46140</v>
-      </c>
-      <c r="D74" s="7">
-        <v>46140</v>
-      </c>
-      <c r="E74" s="7">
-        <v>46100</v>
-      </c>
-      <c r="F74" s="8">
-        <v>4</v>
-      </c>
-      <c r="G74" s="8">
-        <v>4</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J74" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="K74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L74" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="M74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N74" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="O74" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="P74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q74" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="R74" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="S74" s="9">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="75" ht="23" customHeight="1">
-      <c r="A75" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B75" s="7">
-        <v>46142</v>
-      </c>
-      <c r="C75" s="7">
-        <v>45930</v>
-      </c>
-      <c r="D75" s="7">
-        <v>46142</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F75" s="8">
-        <v>6</v>
-      </c>
-      <c r="G75" s="8">
-        <v>6</v>
-      </c>
-      <c r="H75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="K75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L75" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="M75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="N75" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="O75" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="P75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="R75" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="S75" s="9">
-        <v>185.5</v>
-      </c>
-    </row>
-    <row r="76" ht="23" customHeight="1">
-      <c r="A76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B76" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D76" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E76" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F76" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="G76" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="I76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="J76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="K76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="L76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="M76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="N76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="O76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="R76" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="S76" s="13">
-        <f>SUM(S6:S75)</f>
+      <c r="A74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D74" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E74" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F74" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G74" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="J74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="N74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="R74" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="S74" s="13">
+        <f>SUM(S6:S73)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: atualiza template CONTAS-A-RECEBER.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docx_templates/CONTAS-A-RECEBER.xlsx
+++ b/docx_templates/CONTAS-A-RECEBER.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -40,7 +40,7 @@
     </r>
   </si>
   <si>
-    <t>Relatório exportado em quarta-feira, 29 de abril de 2026 por KAROL MEDEIROS</t>
+    <t>Relatório exportado em quinta-feira, 30 de abril de 2026 por KAROL MEDEIROS</t>
   </si>
   <si>
     <t>Conta de Recebimento</t>
@@ -106,15 +106,18 @@
     <t/>
   </si>
   <si>
+    <t>VENCIDO ENTRE 31 A 90 DIAS</t>
+  </si>
+  <si>
+    <t>ANA CONCEIÇÃO CARNEIRO DE ALBUQUERQUE</t>
+  </si>
+  <si>
+    <t>VENCIDO</t>
+  </si>
+  <si>
     <t>VENCIDO ATÉ 30 DIAS</t>
   </si>
   <si>
-    <t>ANA CONCEIÇÃO CARNEIRO DE ALBUQUERQUE</t>
-  </si>
-  <si>
-    <t>VENCIDO</t>
-  </si>
-  <si>
     <t>FA-11240</t>
   </si>
   <si>
@@ -337,22 +340,16 @@
     <t>RAMON TALLES BARBALHO DE FRANÇA</t>
   </si>
   <si>
-    <t>VENCIDO ENTRE 31 A 90 DIAS</t>
-  </si>
-  <si>
     <t>FA-11155</t>
   </si>
   <si>
+    <t>FA-11419</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
+  </si>
+  <si>
     <t>HOJE</t>
-  </si>
-  <si>
-    <t>FA-11419</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
-  </si>
-  <si>
-    <t>A VENCER</t>
   </si>
 </sst>
 </file>
@@ -612,10 +609,10 @@
         <v>23</v>
       </c>
       <c r="F6" s="8">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="G6" s="8">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>24</v>
@@ -671,28 +668,28 @@
         <v>46086</v>
       </c>
       <c r="F7" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G7" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>26</v>
@@ -704,10 +701,10 @@
         <v>23</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S7" s="9">
         <v>620</v>
@@ -730,28 +727,28 @@
         <v>46113</v>
       </c>
       <c r="F8" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G8" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K8" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>26</v>
@@ -763,10 +760,10 @@
         <v>23</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S8" s="9">
         <v>680</v>
@@ -789,16 +786,16 @@
         <v>23</v>
       </c>
       <c r="F9" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G9" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>23</v>
@@ -807,7 +804,7 @@
         <v>23</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>23</v>
@@ -825,7 +822,7 @@
         <v>23</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S9" s="9">
         <v>260</v>
@@ -848,25 +845,25 @@
         <v>23</v>
       </c>
       <c r="F10" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G10" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M10" s="6" t="s">
         <v>23</v>
@@ -878,13 +875,13 @@
         <v>26</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q10" s="6" t="s">
         <v>23</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S10" s="9">
         <v>91.54</v>
@@ -907,25 +904,25 @@
         <v>46118</v>
       </c>
       <c r="F11" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G11" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M11" s="6" t="s">
         <v>23</v>
@@ -940,10 +937,10 @@
         <v>23</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S11" s="9">
         <v>620</v>
@@ -966,28 +963,28 @@
         <v>46086</v>
       </c>
       <c r="F12" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G12" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N12" s="6" t="s">
         <v>26</v>
@@ -999,10 +996,10 @@
         <v>23</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S12" s="9">
         <v>620</v>
@@ -1025,28 +1022,28 @@
         <v>46119</v>
       </c>
       <c r="F13" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G13" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K13" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>26</v>
@@ -1058,10 +1055,10 @@
         <v>23</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S13" s="9">
         <v>620</v>
@@ -1084,25 +1081,25 @@
         <v>46057</v>
       </c>
       <c r="F14" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G14" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K14" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>23</v>
@@ -1117,10 +1114,10 @@
         <v>23</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S14" s="9">
         <v>650</v>
@@ -1143,25 +1140,25 @@
         <v>46118</v>
       </c>
       <c r="F15" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G15" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>23</v>
@@ -1176,10 +1173,10 @@
         <v>23</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S15" s="9">
         <v>680</v>
@@ -1202,28 +1199,28 @@
         <v>46113</v>
       </c>
       <c r="F16" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G16" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>26</v>
@@ -1235,10 +1232,10 @@
         <v>23</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S16" s="9">
         <v>680</v>
@@ -1261,25 +1258,25 @@
         <v>46087</v>
       </c>
       <c r="F17" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G17" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>23</v>
@@ -1294,10 +1291,10 @@
         <v>23</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S17" s="9">
         <v>680</v>
@@ -1320,25 +1317,25 @@
         <v>46127</v>
       </c>
       <c r="F18" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G18" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M18" s="6" t="s">
         <v>23</v>
@@ -1350,13 +1347,13 @@
         <v>26</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S18" s="9">
         <v>680</v>
@@ -1379,25 +1376,25 @@
         <v>23</v>
       </c>
       <c r="F19" s="8">
+        <v>-10</v>
+      </c>
+      <c r="G19" s="8">
         <v>-9</v>
       </c>
-      <c r="G19" s="8">
-        <v>-8</v>
-      </c>
       <c r="H19" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M19" s="6" t="s">
         <v>23</v>
@@ -1415,7 +1412,7 @@
         <v>23</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S19" s="9">
         <v>107.71</v>
@@ -1438,25 +1435,25 @@
         <v>23</v>
       </c>
       <c r="F20" s="8">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="G20" s="8">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>24</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M20" s="6" t="s">
         <v>23</v>
@@ -1474,7 +1471,7 @@
         <v>23</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S20" s="9">
         <v>321.17</v>
@@ -1497,26 +1494,26 @@
         <v>23</v>
       </c>
       <c r="F21" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G21" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K21" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="M21" s="6" t="s">
         <v>23</v>
       </c>
@@ -1533,7 +1530,7 @@
         <v>23</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S21" s="9">
         <v>79.05</v>
@@ -1556,28 +1553,28 @@
         <v>23</v>
       </c>
       <c r="F22" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G22" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K22" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N22" s="6" t="s">
         <v>26</v>
@@ -1592,7 +1589,7 @@
         <v>23</v>
       </c>
       <c r="R22" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S22" s="9">
         <v>200</v>
@@ -1615,25 +1612,25 @@
         <v>23</v>
       </c>
       <c r="F23" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G23" s="8">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M23" s="6" t="s">
         <v>23</v>
@@ -1651,7 +1648,7 @@
         <v>23</v>
       </c>
       <c r="R23" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S23" s="9">
         <v>550</v>
@@ -1674,25 +1671,25 @@
         <v>23</v>
       </c>
       <c r="F24" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G24" s="8">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K24" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M24" s="6" t="s">
         <v>23</v>
@@ -1704,13 +1701,13 @@
         <v>26</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q24" s="6" t="s">
         <v>23</v>
       </c>
       <c r="R24" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S24" s="9">
         <v>650</v>
@@ -1733,25 +1730,25 @@
         <v>23</v>
       </c>
       <c r="F25" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G25" s="8">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M25" s="6" t="s">
         <v>23</v>
@@ -1769,7 +1766,7 @@
         <v>23</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S25" s="9">
         <v>100</v>
@@ -1792,25 +1789,25 @@
         <v>23</v>
       </c>
       <c r="F26" s="8">
-        <v>-30</v>
+        <v>-31</v>
       </c>
       <c r="G26" s="8">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>24</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K26" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M26" s="6" t="s">
         <v>23</v>
@@ -1828,7 +1825,7 @@
         <v>23</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S26" s="9">
         <v>180</v>
@@ -1851,25 +1848,25 @@
         <v>23</v>
       </c>
       <c r="F27" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G27" s="8">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>23</v>
@@ -1887,7 +1884,7 @@
         <v>23</v>
       </c>
       <c r="R27" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S27" s="9">
         <v>302.72</v>
@@ -1910,25 +1907,25 @@
         <v>46127</v>
       </c>
       <c r="F28" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G28" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M28" s="6" t="s">
         <v>23</v>
@@ -1940,13 +1937,13 @@
         <v>26</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R28" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S28" s="9">
         <v>97.15</v>
@@ -1969,26 +1966,26 @@
         <v>46097</v>
       </c>
       <c r="F29" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G29" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J29" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L29" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K29" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="M29" s="6" t="s">
         <v>23</v>
       </c>
@@ -2002,10 +1999,10 @@
         <v>23</v>
       </c>
       <c r="Q29" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R29" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S29" s="9">
         <v>146.55</v>
@@ -2028,25 +2025,25 @@
         <v>23</v>
       </c>
       <c r="F30" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G30" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="K30" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M30" s="6" t="s">
         <v>23</v>
@@ -2064,7 +2061,7 @@
         <v>23</v>
       </c>
       <c r="R30" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S30" s="9">
         <v>154.92</v>
@@ -2087,25 +2084,25 @@
         <v>23</v>
       </c>
       <c r="F31" s="8">
-        <v>-203</v>
+        <v>-204</v>
       </c>
       <c r="G31" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M31" s="6" t="s">
         <v>23</v>
@@ -2123,7 +2120,7 @@
         <v>23</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S31" s="9">
         <v>426</v>
@@ -2146,25 +2143,25 @@
         <v>23</v>
       </c>
       <c r="F32" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G32" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M32" s="6" t="s">
         <v>23</v>
@@ -2182,7 +2179,7 @@
         <v>23</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S32" s="9">
         <v>500</v>
@@ -2205,28 +2202,28 @@
         <v>46127</v>
       </c>
       <c r="F33" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G33" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K33" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N33" s="6" t="s">
         <v>26</v>
@@ -2238,10 +2235,10 @@
         <v>23</v>
       </c>
       <c r="Q33" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S33" s="9">
         <v>600</v>
@@ -2264,28 +2261,28 @@
         <v>46119</v>
       </c>
       <c r="F34" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G34" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K34" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>26</v>
@@ -2297,10 +2294,10 @@
         <v>23</v>
       </c>
       <c r="Q34" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S34" s="9">
         <v>600</v>
@@ -2323,28 +2320,28 @@
         <v>46141</v>
       </c>
       <c r="F35" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G35" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N35" s="6" t="s">
         <v>26</v>
@@ -2356,10 +2353,10 @@
         <v>23</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R35" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S35" s="9">
         <v>620</v>
@@ -2382,25 +2379,25 @@
         <v>46141</v>
       </c>
       <c r="F36" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G36" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>23</v>
@@ -2415,10 +2412,10 @@
         <v>23</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R36" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S36" s="9">
         <v>620</v>
@@ -2441,28 +2438,28 @@
         <v>46119</v>
       </c>
       <c r="F37" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G37" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N37" s="6" t="s">
         <v>26</v>
@@ -2474,10 +2471,10 @@
         <v>23</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R37" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S37" s="9">
         <v>620</v>
@@ -2500,25 +2497,25 @@
         <v>46100</v>
       </c>
       <c r="F38" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>23</v>
@@ -2533,10 +2530,10 @@
         <v>23</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R38" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S38" s="9">
         <v>630</v>
@@ -2559,25 +2556,25 @@
         <v>46112</v>
       </c>
       <c r="F39" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G39" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K39" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>23</v>
@@ -2592,10 +2589,10 @@
         <v>23</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R39" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S39" s="9">
         <v>630</v>
@@ -2618,28 +2615,28 @@
         <v>46119</v>
       </c>
       <c r="F40" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N40" s="6" t="s">
         <v>26</v>
@@ -2651,10 +2648,10 @@
         <v>23</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S40" s="9">
         <v>650</v>
@@ -2677,25 +2674,25 @@
         <v>46122</v>
       </c>
       <c r="F41" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G41" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K41" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>23</v>
@@ -2710,10 +2707,10 @@
         <v>23</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R41" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S41" s="9">
         <v>650</v>
@@ -2736,25 +2733,25 @@
         <v>46119</v>
       </c>
       <c r="F42" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G42" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K42" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M42" s="6" t="s">
         <v>23</v>
@@ -2769,10 +2766,10 @@
         <v>23</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S42" s="9">
         <v>680</v>
@@ -2795,25 +2792,25 @@
         <v>46141</v>
       </c>
       <c r="F43" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K43" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="M43" s="6" t="s">
         <v>23</v>
@@ -2828,10 +2825,10 @@
         <v>23</v>
       </c>
       <c r="Q43" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R43" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S43" s="9">
         <v>680</v>
@@ -2854,28 +2851,28 @@
         <v>46113</v>
       </c>
       <c r="F44" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G44" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K44" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N44" s="6" t="s">
         <v>26</v>
@@ -2887,10 +2884,10 @@
         <v>23</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R44" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S44" s="9">
         <v>680</v>
@@ -2913,25 +2910,25 @@
         <v>46119</v>
       </c>
       <c r="F45" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G45" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>23</v>
@@ -2946,10 +2943,10 @@
         <v>23</v>
       </c>
       <c r="Q45" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R45" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S45" s="9">
         <v>680</v>
@@ -2972,25 +2969,25 @@
         <v>46119</v>
       </c>
       <c r="F46" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G46" s="8">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M46" s="6" t="s">
         <v>23</v>
@@ -3002,13 +2999,13 @@
         <v>26</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q46" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R46" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S46" s="9">
         <v>700</v>
@@ -3031,26 +3028,26 @@
         <v>23</v>
       </c>
       <c r="F47" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G47" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J47" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L47" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K47" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L47" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="M47" s="6" t="s">
         <v>23</v>
       </c>
@@ -3067,7 +3064,7 @@
         <v>23</v>
       </c>
       <c r="R47" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S47" s="9">
         <v>104.04</v>
@@ -3090,25 +3087,25 @@
         <v>23</v>
       </c>
       <c r="F48" s="8">
+        <v>-3</v>
+      </c>
+      <c r="G48" s="8">
         <v>-2</v>
       </c>
-      <c r="G48" s="8">
-        <v>-1</v>
-      </c>
       <c r="H48" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M48" s="6" t="s">
         <v>23</v>
@@ -3126,7 +3123,7 @@
         <v>23</v>
       </c>
       <c r="R48" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S48" s="9">
         <v>120</v>
@@ -3149,25 +3146,25 @@
         <v>23</v>
       </c>
       <c r="F49" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G49" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K49" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M49" s="6" t="s">
         <v>23</v>
@@ -3185,7 +3182,7 @@
         <v>23</v>
       </c>
       <c r="R49" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S49" s="9">
         <v>124.25</v>
@@ -3208,26 +3205,26 @@
         <v>23</v>
       </c>
       <c r="F50" s="8">
+        <v>-3</v>
+      </c>
+      <c r="G50" s="8">
         <v>-2</v>
       </c>
-      <c r="G50" s="8">
-        <v>-1</v>
-      </c>
       <c r="H50" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J50" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L50" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="K50" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>94</v>
-      </c>
       <c r="M50" s="6" t="s">
         <v>23</v>
       </c>
@@ -3244,7 +3241,7 @@
         <v>23</v>
       </c>
       <c r="R50" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S50" s="9">
         <v>202.27</v>
@@ -3267,25 +3264,25 @@
         <v>23</v>
       </c>
       <c r="F51" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G51" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M51" s="6" t="s">
         <v>23</v>
@@ -3303,7 +3300,7 @@
         <v>23</v>
       </c>
       <c r="R51" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S51" s="9">
         <v>350</v>
@@ -3326,25 +3323,25 @@
         <v>23</v>
       </c>
       <c r="F52" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G52" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K52" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M52" s="6" t="s">
         <v>23</v>
@@ -3362,7 +3359,7 @@
         <v>23</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S52" s="9">
         <v>408.24</v>
@@ -3385,25 +3382,25 @@
         <v>23</v>
       </c>
       <c r="F53" s="8">
-        <v>-16</v>
+        <v>-17</v>
       </c>
       <c r="G53" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M53" s="6" t="s">
         <v>23</v>
@@ -3421,7 +3418,7 @@
         <v>23</v>
       </c>
       <c r="R53" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S53" s="9">
         <v>580</v>
@@ -3444,25 +3441,25 @@
         <v>23</v>
       </c>
       <c r="F54" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G54" s="8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>23</v>
@@ -3480,7 +3477,7 @@
         <v>23</v>
       </c>
       <c r="R54" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S54" s="9">
         <v>590</v>
@@ -3503,16 +3500,16 @@
         <v>23</v>
       </c>
       <c r="F55" s="8">
-        <v>-37</v>
+        <v>-38</v>
       </c>
       <c r="G55" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>101</v>
+        <v>24</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>102</v>
@@ -3521,7 +3518,7 @@
         <v>23</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M55" s="6" t="s">
         <v>23</v>
@@ -3530,7 +3527,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>103</v>
+        <v>26</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>23</v>
@@ -3539,7 +3536,7 @@
         <v>23</v>
       </c>
       <c r="R55" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S55" s="9">
         <v>151.25</v>
@@ -3562,25 +3559,25 @@
         <v>23</v>
       </c>
       <c r="F56" s="8">
-        <v>-23</v>
+        <v>-24</v>
       </c>
       <c r="G56" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>23</v>
@@ -3589,7 +3586,7 @@
         <v>26</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>103</v>
+        <v>26</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>23</v>
@@ -3598,7 +3595,7 @@
         <v>23</v>
       </c>
       <c r="R56" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S56" s="9">
         <v>200</v>
@@ -3621,34 +3618,34 @@
         <v>23</v>
       </c>
       <c r="F57" s="8">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="G57" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N57" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>103</v>
+        <v>26</v>
       </c>
       <c r="P57" s="6" t="s">
         <v>23</v>
@@ -3657,7 +3654,7 @@
         <v>23</v>
       </c>
       <c r="R57" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S57" s="9">
         <v>626.62</v>
@@ -3680,10 +3677,10 @@
         <v>23</v>
       </c>
       <c r="F58" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>23</v>
@@ -3704,10 +3701,10 @@
         <v>23</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
chore: atualiza planilha CONTAS-A-RECEBER
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docx_templates/CONTAS-A-RECEBER.xlsx
+++ b/docx_templates/CONTAS-A-RECEBER.xlsx
@@ -40,7 +40,7 @@
     </r>
   </si>
   <si>
-    <t>Relatório exportado em segunda-feira, 11 de maio de 2026 por KAROL MEDEIROS</t>
+    <t>Relatório exportado em terça-feira, 12 de maio de 2026 por KAROL MEDEIROS</t>
   </si>
   <si>
     <t>Conta de Recebimento</t>
@@ -199,226 +199,226 @@
     <t>DAVI HENRIQUE DANTAS DE SOUZA</t>
   </si>
   <si>
+    <t>FA-11255</t>
+  </si>
+  <si>
+    <t>FA-11461</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11460</t>
+  </si>
+  <si>
+    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
+  </si>
+  <si>
+    <t>FA-11356</t>
+  </si>
+  <si>
+    <t>ANDERSON QUEIROZ PINHEIRO</t>
+  </si>
+  <si>
+    <t>FA-11458</t>
+  </si>
+  <si>
+    <t>VENCIDO ACIMA DE 90 DIAS</t>
+  </si>
+  <si>
+    <t>ND-10427</t>
+  </si>
+  <si>
+    <t>RICARDO ARAUJO DE MIRANDA</t>
+  </si>
+  <si>
+    <t>FA-11464</t>
+  </si>
+  <si>
+    <t>FA-11555</t>
+  </si>
+  <si>
+    <t>FA-11553</t>
+  </si>
+  <si>
+    <t>YURI BATISTA DA COSTA</t>
+  </si>
+  <si>
+    <t>FA-11396</t>
+  </si>
+  <si>
+    <t>FA-11466</t>
+  </si>
+  <si>
+    <t>FA-11424</t>
+  </si>
+  <si>
+    <t>OLIZIEL DA SILVA CARDOSO</t>
+  </si>
+  <si>
+    <t>FA-11468</t>
+  </si>
+  <si>
+    <t>FA-11351</t>
+  </si>
+  <si>
+    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
+  </si>
+  <si>
+    <t>FA-11354</t>
+  </si>
+  <si>
+    <t>FA-11614</t>
+  </si>
+  <si>
+    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11587</t>
+  </si>
+  <si>
+    <t>JACKSON CASSIANO VERISSIMO</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA LTDA</t>
+  </si>
+  <si>
+    <t>FA-11114</t>
+  </si>
+  <si>
+    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
+  </si>
+  <si>
+    <t>FA-11355</t>
+  </si>
+  <si>
+    <t>FA-11496</t>
+  </si>
+  <si>
+    <t>FA-11618</t>
+  </si>
+  <si>
+    <t>DANILO DE ALMEIDA TORRES</t>
+  </si>
+  <si>
+    <t>FA-11397</t>
+  </si>
+  <si>
+    <t>JOZILDO TARQUINO DE BRITO</t>
+  </si>
+  <si>
+    <t>FA-11471</t>
+  </si>
+  <si>
+    <t>FA-11522</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11557</t>
+  </si>
+  <si>
+    <t>FA-11556</t>
+  </si>
+  <si>
+    <t>FA-11476</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11398</t>
+  </si>
+  <si>
+    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
+  </si>
+  <si>
+    <t>FA-11399</t>
+  </si>
+  <si>
+    <t>FA-11492</t>
+  </si>
+  <si>
+    <t>ROSSILY PEREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11523</t>
+  </si>
+  <si>
+    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11615</t>
+  </si>
+  <si>
+    <t>FA-11502</t>
+  </si>
+  <si>
+    <t>WESCLY JEAN DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>FA-11473</t>
+  </si>
+  <si>
+    <t>FA-11278</t>
+  </si>
+  <si>
+    <t>FELIPE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11432</t>
+  </si>
+  <si>
+    <t>RAYANE ROBERTA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11475</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11478</t>
+  </si>
+  <si>
+    <t>FA-11558</t>
+  </si>
+  <si>
+    <t>ELSON VIEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11472</t>
+  </si>
+  <si>
+    <t>FA-11327</t>
+  </si>
+  <si>
+    <t>MAICON LOPES SILVA</t>
+  </si>
+  <si>
+    <t>FA-11267</t>
+  </si>
+  <si>
+    <t>ANNY KATARINA ACIOLE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11599</t>
+  </si>
+  <si>
+    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>FA-11575</t>
+  </si>
+  <si>
+    <t>ADRIANO TEOTONIO DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11453</t>
+  </si>
+  <si>
     <t>HOJE</t>
-  </si>
-  <si>
-    <t>FA-11255</t>
-  </si>
-  <si>
-    <t>FA-11461</t>
-  </si>
-  <si>
-    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11460</t>
-  </si>
-  <si>
-    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
-  </si>
-  <si>
-    <t>FA-11356</t>
-  </si>
-  <si>
-    <t>ANDERSON QUEIROZ PINHEIRO</t>
-  </si>
-  <si>
-    <t>FA-11458</t>
-  </si>
-  <si>
-    <t>VENCIDO ACIMA DE 90 DIAS</t>
-  </si>
-  <si>
-    <t>ND-10427</t>
-  </si>
-  <si>
-    <t>RICARDO ARAUJO DE MIRANDA</t>
-  </si>
-  <si>
-    <t>FA-11464</t>
-  </si>
-  <si>
-    <t>FA-11555</t>
-  </si>
-  <si>
-    <t>FA-11553</t>
-  </si>
-  <si>
-    <t>YURI BATISTA DA COSTA</t>
-  </si>
-  <si>
-    <t>FA-11396</t>
-  </si>
-  <si>
-    <t>FA-11466</t>
-  </si>
-  <si>
-    <t>FA-11424</t>
-  </si>
-  <si>
-    <t>OLIZIEL DA SILVA CARDOSO</t>
-  </si>
-  <si>
-    <t>FA-11468</t>
-  </si>
-  <si>
-    <t>FA-11351</t>
-  </si>
-  <si>
-    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
-  </si>
-  <si>
-    <t>FA-11354</t>
-  </si>
-  <si>
-    <t>FA-11614</t>
-  </si>
-  <si>
-    <t>LUCAS SANTOS REVOREDO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11587</t>
-  </si>
-  <si>
-    <t>JACKSON CASSIANO VERISSIMO</t>
-  </si>
-  <si>
-    <t>LUZ DIVINA LTDA</t>
-  </si>
-  <si>
-    <t>FA-11114</t>
-  </si>
-  <si>
-    <t>NICOLAS JUAN HENRIQUE SILVA DE MARIA</t>
-  </si>
-  <si>
-    <t>FA-11355</t>
-  </si>
-  <si>
-    <t>FA-11496</t>
-  </si>
-  <si>
-    <t>FA-11618</t>
-  </si>
-  <si>
-    <t>DANILO DE ALMEIDA TORRES</t>
-  </si>
-  <si>
-    <t>FA-11397</t>
-  </si>
-  <si>
-    <t>JOZILDO TARQUINO DE BRITO</t>
-  </si>
-  <si>
-    <t>FA-11471</t>
-  </si>
-  <si>
-    <t>FA-11522</t>
-  </si>
-  <si>
-    <t>ROBERTO MURATORI</t>
-  </si>
-  <si>
-    <t>FA-11557</t>
-  </si>
-  <si>
-    <t>FA-11556</t>
-  </si>
-  <si>
-    <t>FA-11476</t>
-  </si>
-  <si>
-    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
-  </si>
-  <si>
-    <t>FA-11398</t>
-  </si>
-  <si>
-    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
-  </si>
-  <si>
-    <t>FA-11399</t>
-  </si>
-  <si>
-    <t>FA-11492</t>
-  </si>
-  <si>
-    <t>ROSSILY PEREIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11523</t>
-  </si>
-  <si>
-    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>FA-11615</t>
-  </si>
-  <si>
-    <t>FA-11502</t>
-  </si>
-  <si>
-    <t>WESCLY JEAN DE MEDEIROS</t>
-  </si>
-  <si>
-    <t>FA-11473</t>
-  </si>
-  <si>
-    <t>FA-11278</t>
-  </si>
-  <si>
-    <t>FELIPE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11432</t>
-  </si>
-  <si>
-    <t>RAYANE ROBERTA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11475</t>
-  </si>
-  <si>
-    <t>LUCAS NAJA MOURA RODRIGUES</t>
-  </si>
-  <si>
-    <t>FA-11478</t>
-  </si>
-  <si>
-    <t>FA-11558</t>
-  </si>
-  <si>
-    <t>ELSON VIEIRA DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11472</t>
-  </si>
-  <si>
-    <t>FA-11327</t>
-  </si>
-  <si>
-    <t>MAICON LOPES SILVA</t>
-  </si>
-  <si>
-    <t>FA-11267</t>
-  </si>
-  <si>
-    <t>ANNY KATARINA ACIOLE DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11599</t>
-  </si>
-  <si>
-    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>FA-11575</t>
-  </si>
-  <si>
-    <t>ADRIANO TEOTONIO DA SILVA</t>
-  </si>
-  <si>
-    <t>FA-11453</t>
   </si>
   <si>
     <t>A VENCER</t>
@@ -831,10 +831,10 @@
         <v>23</v>
       </c>
       <c r="F6" s="8">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="G6" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>24</v>
@@ -890,10 +890,10 @@
         <v>23</v>
       </c>
       <c r="F7" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G7" s="8">
-        <v>-19</v>
+        <v>-20</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>25</v>
@@ -949,10 +949,10 @@
         <v>23</v>
       </c>
       <c r="F8" s="8">
-        <v>-42</v>
+        <v>-43</v>
       </c>
       <c r="G8" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>24</v>
@@ -1008,10 +1008,10 @@
         <v>23</v>
       </c>
       <c r="F9" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G9" s="8">
-        <v>-17</v>
+        <v>-18</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>25</v>
@@ -1067,10 +1067,10 @@
         <v>46127</v>
       </c>
       <c r="F10" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G10" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>25</v>
@@ -1126,10 +1126,10 @@
         <v>46097</v>
       </c>
       <c r="F11" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G11" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>25</v>
@@ -1185,10 +1185,10 @@
         <v>23</v>
       </c>
       <c r="F12" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G12" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>25</v>
@@ -1244,10 +1244,10 @@
         <v>46141</v>
       </c>
       <c r="F13" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G13" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>25</v>
@@ -1303,10 +1303,10 @@
         <v>46122</v>
       </c>
       <c r="F14" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G14" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>25</v>
@@ -1362,10 +1362,10 @@
         <v>23</v>
       </c>
       <c r="F15" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G15" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>25</v>
@@ -1421,10 +1421,10 @@
         <v>23</v>
       </c>
       <c r="F16" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G16" s="8">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>25</v>
@@ -1480,10 +1480,10 @@
         <v>23</v>
       </c>
       <c r="F17" s="8">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="G17" s="8">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>25</v>
@@ -1539,10 +1539,10 @@
         <v>46141</v>
       </c>
       <c r="F18" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G18" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>25</v>
@@ -1598,10 +1598,10 @@
         <v>23</v>
       </c>
       <c r="F19" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G19" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>25</v>
@@ -1657,13 +1657,13 @@
         <v>23</v>
       </c>
       <c r="F20" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G20" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I20" s="6" t="s">
         <v>25</v>
@@ -1681,7 +1681,7 @@
         <v>54</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>28</v>
@@ -1716,10 +1716,10 @@
         <v>23</v>
       </c>
       <c r="F21" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G21" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>25</v>
@@ -1728,7 +1728,7 @@
         <v>25</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>23</v>
@@ -1775,10 +1775,10 @@
         <v>46097</v>
       </c>
       <c r="F22" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G22" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>25</v>
@@ -1834,10 +1834,10 @@
         <v>23</v>
       </c>
       <c r="F23" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G23" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>25</v>
@@ -1846,13 +1846,13 @@
         <v>25</v>
       </c>
       <c r="J23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L23" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L23" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="M23" s="6" t="s">
         <v>23</v>
@@ -1893,10 +1893,10 @@
         <v>23</v>
       </c>
       <c r="F24" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G24" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>25</v>
@@ -1905,16 +1905,16 @@
         <v>25</v>
       </c>
       <c r="J24" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="K24" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="M24" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N24" s="6" t="s">
         <v>28</v>
@@ -1952,10 +1952,10 @@
         <v>23</v>
       </c>
       <c r="F25" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G25" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>25</v>
@@ -1964,13 +1964,13 @@
         <v>25</v>
       </c>
       <c r="J25" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L25" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="M25" s="6" t="s">
         <v>23</v>
@@ -2011,10 +2011,10 @@
         <v>23</v>
       </c>
       <c r="F26" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G26" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>25</v>
@@ -2023,7 +2023,7 @@
         <v>25</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K26" s="6" t="s">
         <v>23</v>
@@ -2070,25 +2070,25 @@
         <v>23</v>
       </c>
       <c r="F27" s="8">
-        <v>-215</v>
+        <v>-216</v>
       </c>
       <c r="G27" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H27" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I27" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J27" s="6" t="s">
+      <c r="K27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L27" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="M27" s="6" t="s">
         <v>23</v>
@@ -2129,10 +2129,10 @@
         <v>46119</v>
       </c>
       <c r="F28" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G28" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>25</v>
@@ -2141,7 +2141,7 @@
         <v>25</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>23</v>
@@ -2188,10 +2188,10 @@
         <v>46141</v>
       </c>
       <c r="F29" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G29" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>25</v>
@@ -2200,7 +2200,7 @@
         <v>25</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>23</v>
@@ -2247,10 +2247,10 @@
         <v>46141</v>
       </c>
       <c r="F30" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G30" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>25</v>
@@ -2259,13 +2259,13 @@
         <v>25</v>
       </c>
       <c r="J30" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L30" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="K30" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L30" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="M30" s="6" t="s">
         <v>23</v>
@@ -2306,10 +2306,10 @@
         <v>46112</v>
       </c>
       <c r="F31" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G31" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>25</v>
@@ -2318,7 +2318,7 @@
         <v>25</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>23</v>
@@ -2365,10 +2365,10 @@
         <v>46119</v>
       </c>
       <c r="F32" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G32" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>25</v>
@@ -2377,16 +2377,16 @@
         <v>25</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N32" s="6" t="s">
         <v>28</v>
@@ -2424,10 +2424,10 @@
         <v>23</v>
       </c>
       <c r="F33" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G33" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>25</v>
@@ -2436,13 +2436,13 @@
         <v>25</v>
       </c>
       <c r="J33" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="K33" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="M33" s="6" t="s">
         <v>23</v>
@@ -2483,10 +2483,10 @@
         <v>46119</v>
       </c>
       <c r="F34" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G34" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>25</v>
@@ -2495,13 +2495,13 @@
         <v>25</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K34" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M34" s="6" t="s">
         <v>23</v>
@@ -2542,10 +2542,10 @@
         <v>23</v>
       </c>
       <c r="F35" s="8">
-        <v>-14</v>
+        <v>-15</v>
       </c>
       <c r="G35" s="8">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>25</v>
@@ -2554,13 +2554,13 @@
         <v>25</v>
       </c>
       <c r="J35" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L35" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="M35" s="6" t="s">
         <v>23</v>
@@ -2601,11 +2601,11 @@
         <v>23</v>
       </c>
       <c r="F36" s="8">
+        <v>-8</v>
+      </c>
+      <c r="G36" s="8">
         <v>-7</v>
       </c>
-      <c r="G36" s="8">
-        <v>-6</v>
-      </c>
       <c r="H36" s="6" t="s">
         <v>25</v>
       </c>
@@ -2613,13 +2613,13 @@
         <v>25</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>23</v>
@@ -2660,10 +2660,10 @@
         <v>23</v>
       </c>
       <c r="F37" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G37" s="8">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>25</v>
@@ -2672,13 +2672,13 @@
         <v>25</v>
       </c>
       <c r="J37" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L37" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="K37" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>23</v>
@@ -2719,10 +2719,10 @@
         <v>46148</v>
       </c>
       <c r="F38" s="8">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="G38" s="8">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>25</v>
@@ -2731,31 +2731,31 @@
         <v>25</v>
       </c>
       <c r="J38" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L38" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="K38" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L38" s="6" t="s">
+      <c r="M38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q38" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="R38" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="M38" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N38" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O38" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P38" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q38" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="R38" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="S38" s="9">
         <v>685.71</v>
@@ -2778,10 +2778,10 @@
         <v>23</v>
       </c>
       <c r="F39" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G39" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>25</v>
@@ -2790,13 +2790,13 @@
         <v>25</v>
       </c>
       <c r="J39" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="K39" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="M39" s="6" t="s">
         <v>23</v>
@@ -2837,10 +2837,10 @@
         <v>23</v>
       </c>
       <c r="F40" s="8">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G40" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>25</v>
@@ -2849,13 +2849,13 @@
         <v>25</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>23</v>
@@ -2896,10 +2896,10 @@
         <v>23</v>
       </c>
       <c r="F41" s="8">
-        <v>-28</v>
+        <v>-29</v>
       </c>
       <c r="G41" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>25</v>
@@ -2908,7 +2908,7 @@
         <v>25</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K41" s="6" t="s">
         <v>23</v>
@@ -2955,10 +2955,10 @@
         <v>46153</v>
       </c>
       <c r="F42" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G42" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>25</v>
@@ -2967,13 +2967,13 @@
         <v>25</v>
       </c>
       <c r="J42" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L42" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="K42" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L42" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="M42" s="6" t="s">
         <v>23</v>
@@ -3014,16 +3014,16 @@
         <v>46097</v>
       </c>
       <c r="F43" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G43" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>31</v>
@@ -3038,10 +3038,10 @@
         <v>23</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P43" s="6" t="s">
         <v>23</v>
@@ -3073,34 +3073,34 @@
         <v>46112</v>
       </c>
       <c r="F44" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G44" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J44" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L44" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="K44" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>91</v>
-      </c>
       <c r="M44" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>23</v>
@@ -3132,19 +3132,19 @@
         <v>46119</v>
       </c>
       <c r="F45" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G45" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>23</v>
@@ -3156,10 +3156,10 @@
         <v>52</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O45" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P45" s="6" t="s">
         <v>23</v>
@@ -3191,34 +3191,34 @@
         <v>46127</v>
       </c>
       <c r="F46" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G46" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J46" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L46" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="K46" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L46" s="6" t="s">
-        <v>94</v>
-      </c>
       <c r="M46" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>23</v>
@@ -3250,34 +3250,34 @@
         <v>46141</v>
       </c>
       <c r="F47" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G47" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K47" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M47" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P47" s="6" t="s">
         <v>23</v>
@@ -3309,19 +3309,19 @@
         <v>46141</v>
       </c>
       <c r="F48" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G48" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>23</v>
@@ -3333,10 +3333,10 @@
         <v>43</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>23</v>
@@ -3368,34 +3368,34 @@
         <v>46119</v>
       </c>
       <c r="F49" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G49" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J49" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L49" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="K49" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L49" s="6" t="s">
-        <v>98</v>
-      </c>
       <c r="M49" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P49" s="6" t="s">
         <v>23</v>
@@ -3427,34 +3427,34 @@
         <v>46112</v>
       </c>
       <c r="F50" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J50" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L50" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="K50" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="M50" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>23</v>
@@ -3486,19 +3486,19 @@
         <v>46112</v>
       </c>
       <c r="F51" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G51" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>23</v>
@@ -3510,10 +3510,10 @@
         <v>23</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P51" s="6" t="s">
         <v>23</v>
@@ -3545,34 +3545,34 @@
         <v>46119</v>
       </c>
       <c r="F52" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G52" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J52" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L52" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="K52" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="M52" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>29</v>
@@ -3604,34 +3604,34 @@
         <v>46127</v>
       </c>
       <c r="F53" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G53" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J53" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L53" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="K53" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L53" s="6" t="s">
-        <v>105</v>
-      </c>
       <c r="M53" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O53" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P53" s="6" t="s">
         <v>23</v>
@@ -3663,34 +3663,34 @@
         <v>46150</v>
       </c>
       <c r="F54" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G54" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>23</v>
@@ -3722,34 +3722,34 @@
         <v>46127</v>
       </c>
       <c r="F55" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G55" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J55" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L55" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="K55" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L55" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="M55" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P55" s="6" t="s">
         <v>23</v>
@@ -3781,34 +3781,34 @@
         <v>46119</v>
       </c>
       <c r="F56" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G56" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>23</v>
@@ -3840,34 +3840,34 @@
         <v>46092</v>
       </c>
       <c r="F57" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G57" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J57" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L57" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="K57" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L57" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="M57" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P57" s="6" t="s">
         <v>23</v>
@@ -3899,34 +3899,34 @@
         <v>46119</v>
       </c>
       <c r="F58" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G58" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J58" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L58" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="K58" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L58" s="6" t="s">
-        <v>113</v>
-      </c>
       <c r="M58" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>23</v>
@@ -3958,34 +3958,34 @@
         <v>46119</v>
       </c>
       <c r="F59" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G59" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J59" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L59" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="K59" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L59" s="6" t="s">
-        <v>115</v>
-      </c>
       <c r="M59" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P59" s="6" t="s">
         <v>23</v>
@@ -4017,19 +4017,19 @@
         <v>46119</v>
       </c>
       <c r="F60" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G60" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K60" s="6" t="s">
         <v>23</v>
@@ -4041,10 +4041,10 @@
         <v>23</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>23</v>
@@ -4076,34 +4076,34 @@
         <v>46141</v>
       </c>
       <c r="F61" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G61" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J61" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L61" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="K61" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L61" s="6" t="s">
-        <v>118</v>
-      </c>
       <c r="M61" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O61" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P61" s="6" t="s">
         <v>23</v>
@@ -4135,34 +4135,34 @@
         <v>46119</v>
       </c>
       <c r="F62" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G62" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M62" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>29</v>
@@ -4194,34 +4194,34 @@
         <v>46099</v>
       </c>
       <c r="F63" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G63" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J63" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L63" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="K63" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L63" s="6" t="s">
-        <v>121</v>
-      </c>
       <c r="M63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O63" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P63" s="6" t="s">
         <v>23</v>
@@ -4253,34 +4253,34 @@
         <v>46092</v>
       </c>
       <c r="F64" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G64" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J64" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L64" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="K64" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L64" s="6" t="s">
-        <v>123</v>
-      </c>
       <c r="M64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>23</v>
@@ -4312,34 +4312,34 @@
         <v>46148</v>
       </c>
       <c r="F65" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G65" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J65" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L65" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="K65" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L65" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="M65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="O65" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P65" s="6" t="s">
         <v>23</v>
@@ -4371,26 +4371,26 @@
         <v>46148</v>
       </c>
       <c r="F66" s="8">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="G66" s="8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J66" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L66" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="K66" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>127</v>
-      </c>
       <c r="M66" s="6" t="s">
         <v>23</v>
       </c>
@@ -4398,7 +4398,7 @@
         <v>28</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>23</v>
@@ -4407,7 +4407,7 @@
         <v>39</v>
       </c>
       <c r="R66" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S66" s="9">
         <v>1028.57</v>
@@ -4430,10 +4430,10 @@
         <v>23</v>
       </c>
       <c r="F67" s="8">
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="G67" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>25</v>
@@ -4442,22 +4442,22 @@
         <v>23</v>
       </c>
       <c r="J67" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L67" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="N67" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O67" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="K67" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L67" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="M67" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="N67" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O67" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="P67" s="6" t="s">
         <v>23</v>
@@ -4489,10 +4489,10 @@
         <v>46097</v>
       </c>
       <c r="F68" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G68" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>23</v>
@@ -4548,10 +4548,10 @@
         <v>46112</v>
       </c>
       <c r="F69" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G69" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H69" s="6" t="s">
         <v>23</v>
@@ -4566,10 +4566,10 @@
         <v>23</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N69" s="6" t="s">
         <v>129</v>
@@ -4607,10 +4607,10 @@
         <v>46119</v>
       </c>
       <c r="F70" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G70" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>23</v>
@@ -4666,10 +4666,10 @@
         <v>46127</v>
       </c>
       <c r="F71" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G71" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>23</v>
@@ -4684,10 +4684,10 @@
         <v>23</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N71" s="6" t="s">
         <v>129</v>
@@ -4725,10 +4725,10 @@
         <v>46119</v>
       </c>
       <c r="F72" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G72" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>23</v>
@@ -4743,10 +4743,10 @@
         <v>23</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N72" s="6" t="s">
         <v>129</v>
@@ -4784,10 +4784,10 @@
         <v>46141</v>
       </c>
       <c r="F73" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G73" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H73" s="6" t="s">
         <v>23</v>
@@ -4802,7 +4802,7 @@
         <v>23</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M73" s="6" t="s">
         <v>23</v>
@@ -4843,10 +4843,10 @@
         <v>46141</v>
       </c>
       <c r="F74" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G74" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>23</v>
@@ -4902,10 +4902,10 @@
         <v>46119</v>
       </c>
       <c r="F75" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G75" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>23</v>
@@ -4920,7 +4920,7 @@
         <v>23</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>23</v>
@@ -4961,10 +4961,10 @@
         <v>46127</v>
       </c>
       <c r="F76" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G76" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H76" s="6" t="s">
         <v>23</v>
@@ -4979,7 +4979,7 @@
         <v>23</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M76" s="6" t="s">
         <v>23</v>
@@ -5020,10 +5020,10 @@
         <v>46112</v>
       </c>
       <c r="F77" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G77" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H77" s="6" t="s">
         <v>23</v>
@@ -5038,7 +5038,7 @@
         <v>23</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M77" s="6" t="s">
         <v>23</v>
@@ -5079,10 +5079,10 @@
         <v>46112</v>
       </c>
       <c r="F78" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G78" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>23</v>
@@ -5138,10 +5138,10 @@
         <v>46150</v>
       </c>
       <c r="F79" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G79" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>23</v>
@@ -5156,7 +5156,7 @@
         <v>23</v>
       </c>
       <c r="L79" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M79" s="6" t="s">
         <v>23</v>
@@ -5197,10 +5197,10 @@
         <v>46153</v>
       </c>
       <c r="F80" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G80" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>23</v>
@@ -5215,7 +5215,7 @@
         <v>23</v>
       </c>
       <c r="L80" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M80" s="6" t="s">
         <v>23</v>
@@ -5256,10 +5256,10 @@
         <v>46092</v>
       </c>
       <c r="F81" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G81" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H81" s="6" t="s">
         <v>23</v>
@@ -5274,7 +5274,7 @@
         <v>23</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M81" s="6" t="s">
         <v>23</v>
@@ -5315,10 +5315,10 @@
         <v>46127</v>
       </c>
       <c r="F82" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G82" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>23</v>
@@ -5333,7 +5333,7 @@
         <v>23</v>
       </c>
       <c r="L82" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M82" s="6" t="s">
         <v>23</v>
@@ -5374,10 +5374,10 @@
         <v>46119</v>
       </c>
       <c r="F83" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G83" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H83" s="6" t="s">
         <v>23</v>
@@ -5392,10 +5392,10 @@
         <v>23</v>
       </c>
       <c r="L83" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M83" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N83" s="6" t="s">
         <v>129</v>
@@ -5433,10 +5433,10 @@
         <v>46119</v>
       </c>
       <c r="F84" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G84" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H84" s="6" t="s">
         <v>23</v>
@@ -5451,7 +5451,7 @@
         <v>23</v>
       </c>
       <c r="L84" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M84" s="6" t="s">
         <v>23</v>
@@ -5492,10 +5492,10 @@
         <v>46113</v>
       </c>
       <c r="F85" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G85" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H85" s="6" t="s">
         <v>23</v>
@@ -5551,10 +5551,10 @@
         <v>46119</v>
       </c>
       <c r="F86" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G86" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H86" s="6" t="s">
         <v>23</v>
@@ -5569,7 +5569,7 @@
         <v>23</v>
       </c>
       <c r="L86" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M86" s="6" t="s">
         <v>23</v>
@@ -5610,10 +5610,10 @@
         <v>46119</v>
       </c>
       <c r="F87" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G87" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>23</v>
@@ -5669,10 +5669,10 @@
         <v>46141</v>
       </c>
       <c r="F88" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G88" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>23</v>
@@ -5687,7 +5687,7 @@
         <v>23</v>
       </c>
       <c r="L88" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M88" s="6" t="s">
         <v>23</v>
@@ -5728,10 +5728,10 @@
         <v>46092</v>
       </c>
       <c r="F89" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G89" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>23</v>
@@ -5746,7 +5746,7 @@
         <v>23</v>
       </c>
       <c r="L89" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>23</v>
@@ -5787,10 +5787,10 @@
         <v>46099</v>
       </c>
       <c r="F90" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G90" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H90" s="6" t="s">
         <v>23</v>
@@ -5805,7 +5805,7 @@
         <v>23</v>
       </c>
       <c r="L90" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M90" s="6" t="s">
         <v>23</v>
@@ -5846,10 +5846,10 @@
         <v>46119</v>
       </c>
       <c r="F91" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G91" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H91" s="6" t="s">
         <v>23</v>
@@ -5864,7 +5864,7 @@
         <v>23</v>
       </c>
       <c r="L91" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M91" s="6" t="s">
         <v>23</v>
@@ -5905,10 +5905,10 @@
         <v>46148</v>
       </c>
       <c r="F92" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G92" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H92" s="6" t="s">
         <v>23</v>
@@ -5923,7 +5923,7 @@
         <v>23</v>
       </c>
       <c r="L92" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M92" s="6" t="s">
         <v>23</v>
@@ -5964,10 +5964,10 @@
         <v>46148</v>
       </c>
       <c r="F93" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G93" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H93" s="6" t="s">
         <v>23</v>
@@ -5982,25 +5982,25 @@
         <v>23</v>
       </c>
       <c r="L93" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N93" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="O93" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="P93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q93" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="R93" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="M93" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N93" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="O93" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="P93" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q93" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="R93" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="S93" s="9">
         <v>1200</v>
@@ -6023,10 +6023,10 @@
         <v>46148</v>
       </c>
       <c r="F94" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G94" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H94" s="6" t="s">
         <v>23</v>
@@ -6041,7 +6041,7 @@
         <v>23</v>
       </c>
       <c r="L94" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M94" s="6" t="s">
         <v>23</v>
@@ -6059,7 +6059,7 @@
         <v>39</v>
       </c>
       <c r="R94" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S94" s="9">
         <v>1200</v>
@@ -6082,10 +6082,10 @@
         <v>46149</v>
       </c>
       <c r="F95" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G95" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H95" s="6" t="s">
         <v>25</v>
@@ -6141,10 +6141,10 @@
         <v>46097</v>
       </c>
       <c r="F96" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G96" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H96" s="6" t="s">
         <v>23</v>
@@ -6200,10 +6200,10 @@
         <v>46119</v>
       </c>
       <c r="F97" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G97" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H97" s="6" t="s">
         <v>23</v>
@@ -6259,10 +6259,10 @@
         <v>46141</v>
       </c>
       <c r="F98" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G98" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H98" s="6" t="s">
         <v>23</v>
@@ -6277,7 +6277,7 @@
         <v>23</v>
       </c>
       <c r="L98" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M98" s="6" t="s">
         <v>23</v>
@@ -6318,10 +6318,10 @@
         <v>46141</v>
       </c>
       <c r="F99" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G99" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H99" s="6" t="s">
         <v>23</v>
@@ -6377,10 +6377,10 @@
         <v>46119</v>
       </c>
       <c r="F100" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G100" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H100" s="6" t="s">
         <v>23</v>
@@ -6395,10 +6395,10 @@
         <v>23</v>
       </c>
       <c r="L100" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M100" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N100" s="6" t="s">
         <v>129</v>
@@ -6436,10 +6436,10 @@
         <v>46119</v>
       </c>
       <c r="F101" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G101" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H101" s="6" t="s">
         <v>23</v>
@@ -6454,7 +6454,7 @@
         <v>23</v>
       </c>
       <c r="L101" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M101" s="6" t="s">
         <v>23</v>
@@ -6495,10 +6495,10 @@
         <v>46150</v>
       </c>
       <c r="F102" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G102" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H102" s="6" t="s">
         <v>23</v>
@@ -6513,7 +6513,7 @@
         <v>23</v>
       </c>
       <c r="L102" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M102" s="6" t="s">
         <v>23</v>
@@ -6554,10 +6554,10 @@
         <v>46153</v>
       </c>
       <c r="F103" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G103" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H103" s="6" t="s">
         <v>23</v>
@@ -6572,7 +6572,7 @@
         <v>23</v>
       </c>
       <c r="L103" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M103" s="6" t="s">
         <v>23</v>
@@ -6613,10 +6613,10 @@
         <v>46119</v>
       </c>
       <c r="F104" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G104" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H104" s="6" t="s">
         <v>23</v>
@@ -6631,10 +6631,10 @@
         <v>23</v>
       </c>
       <c r="L104" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M104" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N104" s="6" t="s">
         <v>129</v>
@@ -6672,10 +6672,10 @@
         <v>46127</v>
       </c>
       <c r="F105" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G105" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H105" s="6" t="s">
         <v>23</v>
@@ -6690,7 +6690,7 @@
         <v>23</v>
       </c>
       <c r="L105" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M105" s="6" t="s">
         <v>23</v>
@@ -6731,10 +6731,10 @@
         <v>46092</v>
       </c>
       <c r="F106" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G106" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H106" s="6" t="s">
         <v>23</v>
@@ -6749,7 +6749,7 @@
         <v>23</v>
       </c>
       <c r="L106" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M106" s="6" t="s">
         <v>23</v>
@@ -6790,10 +6790,10 @@
         <v>46119</v>
       </c>
       <c r="F107" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G107" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H107" s="6" t="s">
         <v>23</v>
@@ -6808,7 +6808,7 @@
         <v>23</v>
       </c>
       <c r="L107" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M107" s="6" t="s">
         <v>23</v>
@@ -6849,10 +6849,10 @@
         <v>46113</v>
       </c>
       <c r="F108" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G108" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H108" s="6" t="s">
         <v>23</v>
@@ -6908,10 +6908,10 @@
         <v>46119</v>
       </c>
       <c r="F109" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G109" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H109" s="6" t="s">
         <v>23</v>
@@ -6926,7 +6926,7 @@
         <v>23</v>
       </c>
       <c r="L109" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M109" s="6" t="s">
         <v>23</v>
@@ -6967,10 +6967,10 @@
         <v>46119</v>
       </c>
       <c r="F110" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G110" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H110" s="6" t="s">
         <v>23</v>
@@ -7026,10 +7026,10 @@
         <v>46141</v>
       </c>
       <c r="F111" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G111" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H111" s="6" t="s">
         <v>23</v>
@@ -7044,7 +7044,7 @@
         <v>23</v>
       </c>
       <c r="L111" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M111" s="6" t="s">
         <v>23</v>
@@ -7085,10 +7085,10 @@
         <v>46099</v>
       </c>
       <c r="F112" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G112" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H112" s="6" t="s">
         <v>23</v>
@@ -7103,7 +7103,7 @@
         <v>23</v>
       </c>
       <c r="L112" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M112" s="6" t="s">
         <v>23</v>
@@ -7144,10 +7144,10 @@
         <v>46148</v>
       </c>
       <c r="F113" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G113" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H113" s="6" t="s">
         <v>23</v>
@@ -7162,7 +7162,7 @@
         <v>23</v>
       </c>
       <c r="L113" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="M113" s="6" t="s">
         <v>23</v>
@@ -7203,10 +7203,10 @@
         <v>46148</v>
       </c>
       <c r="F114" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G114" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H114" s="6" t="s">
         <v>23</v>
@@ -7221,25 +7221,25 @@
         <v>23</v>
       </c>
       <c r="L114" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M114" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N114" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="O114" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="P114" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q114" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="R114" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="M114" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N114" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="O114" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="P114" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q114" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="R114" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="S114" s="9">
         <v>1200</v>
@@ -7262,10 +7262,10 @@
         <v>46148</v>
       </c>
       <c r="F115" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G115" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H115" s="6" t="s">
         <v>23</v>
@@ -7280,7 +7280,7 @@
         <v>23</v>
       </c>
       <c r="L115" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M115" s="6" t="s">
         <v>23</v>
@@ -7298,7 +7298,7 @@
         <v>39</v>
       </c>
       <c r="R115" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S115" s="9">
         <v>1200</v>
@@ -7321,10 +7321,10 @@
         <v>46149</v>
       </c>
       <c r="F116" s="8">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="G116" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H116" s="6" t="s">
         <v>25</v>
@@ -7380,10 +7380,10 @@
         <v>23</v>
       </c>
       <c r="F117" s="8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G117" s="8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H117" s="6" t="s">
         <v>23</v>

</xml_diff>